<commit_message>
run again for average metrics as well
</commit_message>
<xml_diff>
--- a/dataset_agreed/saved_models/hyperparameter_optimized_runs/pointcloud_HPO_run_1/epoch_10/per_file_predictions_epoch_10.xlsx
+++ b/dataset_agreed/saved_models/hyperparameter_optimized_runs/pointcloud_HPO_run_1/epoch_10/per_file_predictions_epoch_10.xlsx
@@ -808,769 +808,769 @@
     <t>0,1,1,0</t>
   </si>
   <si>
-    <t>0.4760,0.1257,0.5051,0.0239</t>
-  </si>
-  <si>
-    <t>0.5412,0.0657,0.2545,0.1308</t>
-  </si>
-  <si>
-    <t>0.5313,0.1146,0.4238,0.0380</t>
-  </si>
-  <si>
-    <t>0.6203,0.0725,0.3040,0.0506</t>
-  </si>
-  <si>
-    <t>0.6768,0.1143,0.2056,0.0350</t>
-  </si>
-  <si>
-    <t>0.5756,0.1441,0.2758,0.0474</t>
-  </si>
-  <si>
-    <t>0.6444,0.0808,0.3250,0.0326</t>
-  </si>
-  <si>
-    <t>0.6733,0.1037,0.2244,0.0341</t>
-  </si>
-  <si>
-    <t>0.6080,0.1405,0.2744,0.0444</t>
-  </si>
-  <si>
-    <t>0.6304,0.1625,0.2258,0.0272</t>
-  </si>
-  <si>
-    <t>0.6317,0.1153,0.2955,0.0274</t>
-  </si>
-  <si>
-    <t>0.5630,0.1772,0.3013,0.0432</t>
-  </si>
-  <si>
-    <t>0.4548,0.0466,0.6039,0.0184</t>
-  </si>
-  <si>
-    <t>0.5255,0.0883,0.4551,0.0255</t>
-  </si>
-  <si>
-    <t>0.4207,0.0924,0.5499,0.0354</t>
-  </si>
-  <si>
-    <t>0.3718,0.0665,0.6600,0.0216</t>
-  </si>
-  <si>
-    <t>0.5523,0.0875,0.3516,0.0604</t>
-  </si>
-  <si>
-    <t>0.2906,0.3499,0.4222,0.0101</t>
-  </si>
-  <si>
-    <t>0.4713,0.1900,0.4189,0.0134</t>
-  </si>
-  <si>
-    <t>0.5956,0.1310,0.3349,0.0192</t>
-  </si>
-  <si>
-    <t>0.4430,0.3353,0.3269,0.0233</t>
-  </si>
-  <si>
-    <t>0.3480,0.3516,0.3972,0.0112</t>
-  </si>
-  <si>
-    <t>0.4654,0.0708,0.5380,0.0209</t>
-  </si>
-  <si>
-    <t>0.3303,0.0552,0.7240,0.0239</t>
-  </si>
-  <si>
-    <t>0.3094,0.0234,0.7949,0.0060</t>
-  </si>
-  <si>
-    <t>0.4350,0.0594,0.5792,0.0268</t>
-  </si>
-  <si>
-    <t>0.2964,0.0440,0.7622,0.0155</t>
-  </si>
-  <si>
-    <t>0.3278,0.0505,0.7326,0.0118</t>
-  </si>
-  <si>
-    <t>0.1002,0.0291,0.9200,0.0101</t>
-  </si>
-  <si>
-    <t>0.5498,0.1432,0.3747,0.0230</t>
-  </si>
-  <si>
-    <t>0.5216,0.1437,0.4142,0.0216</t>
-  </si>
-  <si>
-    <t>0.0175,0.0391,0.9801,0.0028</t>
-  </si>
-  <si>
-    <t>0.3813,0.1676,0.5383,0.0127</t>
-  </si>
-  <si>
-    <t>0.5844,0.1042,0.3470,0.0320</t>
-  </si>
-  <si>
-    <t>0.5713,0.1359,0.3342,0.0363</t>
-  </si>
-  <si>
-    <t>0.5759,0.1337,0.3456,0.0222</t>
-  </si>
-  <si>
-    <t>0.4973,0.1738,0.4181,0.0276</t>
-  </si>
-  <si>
-    <t>0.0649,0.4534,0.7462,0.0164</t>
-  </si>
-  <si>
-    <t>0.2426,0.0513,0.7781,0.0097</t>
-  </si>
-  <si>
-    <t>0.2160,0.0638,0.7919,0.0104</t>
-  </si>
-  <si>
-    <t>0.4022,0.0617,0.6246,0.0214</t>
-  </si>
-  <si>
-    <t>0.2160,0.0901,0.7701,0.0098</t>
-  </si>
-  <si>
-    <t>0.1190,0.7279,0.2612,0.0099</t>
-  </si>
-  <si>
-    <t>0.1922,0.0676,0.8214,0.0177</t>
-  </si>
-  <si>
-    <t>0.5164,0.0942,0.4339,0.0483</t>
-  </si>
-  <si>
-    <t>0.3931,0.2124,0.4858,0.0194</t>
-  </si>
-  <si>
-    <t>0.2043,0.4669,0.4902,0.0129</t>
-  </si>
-  <si>
-    <t>0.4583,0.1407,0.4976,0.0131</t>
-  </si>
-  <si>
-    <t>0.0684,0.1407,0.8783,0.0064</t>
-  </si>
-  <si>
-    <t>0.1763,0.0777,0.8181,0.0055</t>
-  </si>
-  <si>
-    <t>0.3100,0.0894,0.6929,0.0291</t>
-  </si>
-  <si>
-    <t>0.3019,0.0424,0.7365,0.0148</t>
-  </si>
-  <si>
-    <t>0.1504,0.0405,0.8731,0.0090</t>
-  </si>
-  <si>
-    <t>0.1858,0.0501,0.8483,0.0090</t>
-  </si>
-  <si>
-    <t>0.6021,0.1380,0.3111,0.0343</t>
-  </si>
-  <si>
-    <t>0.5945,0.1064,0.3360,0.0346</t>
-  </si>
-  <si>
-    <t>0.6413,0.1169,0.2680,0.0226</t>
-  </si>
-  <si>
-    <t>0.2857,0.1030,0.7091,0.0127</t>
-  </si>
-  <si>
-    <t>0.6880,0.0889,0.2263,0.0294</t>
-  </si>
-  <si>
-    <t>0.6260,0.1128,0.2556,0.0341</t>
-  </si>
-  <si>
-    <t>0.5883,0.1137,0.3495,0.0290</t>
-  </si>
-  <si>
-    <t>0.0453,0.4764,0.7781,0.0061</t>
-  </si>
-  <si>
-    <t>0.0938,0.0586,0.9103,0.0044</t>
-  </si>
-  <si>
-    <t>0.1448,0.0448,0.8809,0.0089</t>
-  </si>
-  <si>
-    <t>0.0801,0.3391,0.7384,0.0069</t>
-  </si>
-  <si>
-    <t>0.1078,0.0319,0.9146,0.0042</t>
-  </si>
-  <si>
-    <t>0.4679,0.1596,0.4399,0.0149</t>
-  </si>
-  <si>
-    <t>0.0393,0.9237,0.1906,0.0039</t>
-  </si>
-  <si>
-    <t>0.5904,0.0999,0.3365,0.0377</t>
-  </si>
-  <si>
-    <t>0.5635,0.1266,0.3735,0.0214</t>
-  </si>
-  <si>
-    <t>0.1470,0.2935,0.7269,0.0081</t>
-  </si>
-  <si>
-    <t>0.0887,0.3198,0.7654,0.0108</t>
-  </si>
-  <si>
-    <t>0.1138,0.3271,0.7070,0.0071</t>
-  </si>
-  <si>
-    <t>0.0598,0.6977,0.5127,0.0051</t>
-  </si>
-  <si>
-    <t>0.1124,0.1656,0.8062,0.0060</t>
-  </si>
-  <si>
-    <t>0.4592,0.0575,0.4089,0.1034</t>
-  </si>
-  <si>
-    <t>0.5669,0.0614,0.3650,0.0511</t>
-  </si>
-  <si>
-    <t>0.6452,0.0501,0.2024,0.0869</t>
-  </si>
-  <si>
-    <t>0.5660,0.0877,0.3627,0.0562</t>
-  </si>
-  <si>
-    <t>0.5417,0.0716,0.3364,0.0762</t>
-  </si>
-  <si>
-    <t>0.5942,0.0372,0.3857,0.0370</t>
-  </si>
-  <si>
-    <t>0.0658,0.5327,0.6711,0.0074</t>
-  </si>
-  <si>
-    <t>0.0693,0.0893,0.9093,0.0041</t>
-  </si>
-  <si>
-    <t>0.1570,0.2289,0.7057,0.0059</t>
-  </si>
-  <si>
-    <t>0.1378,0.1648,0.7798,0.0084</t>
-  </si>
-  <si>
-    <t>0.0452,0.5711,0.7359,0.0042</t>
-  </si>
-  <si>
-    <t>0.1126,0.3781,0.6618,0.0069</t>
-  </si>
-  <si>
-    <t>0.5981,0.1349,0.2519,0.0476</t>
-  </si>
-  <si>
-    <t>0.6735,0.0996,0.2290,0.0338</t>
-  </si>
-  <si>
-    <t>0.4958,0.2028,0.3600,0.0348</t>
-  </si>
-  <si>
-    <t>0.6107,0.1357,0.2248,0.0532</t>
-  </si>
-  <si>
-    <t>0.6751,0.0951,0.2439,0.0168</t>
-  </si>
-  <si>
-    <t>0.6856,0.1049,0.1921,0.0415</t>
-  </si>
-  <si>
-    <t>0.6875,0.0816,0.2561,0.0242</t>
-  </si>
-  <si>
-    <t>0.4757,0.2262,0.3717,0.0327</t>
-  </si>
-  <si>
-    <t>0.6476,0.1387,0.2298,0.0406</t>
-  </si>
-  <si>
-    <t>0.7485,0.0672,0.1338,0.0446</t>
-  </si>
-  <si>
-    <t>0.6861,0.0814,0.1975,0.0469</t>
-  </si>
-  <si>
-    <t>0.6122,0.0991,0.3593,0.0272</t>
-  </si>
-  <si>
-    <t>0.6501,0.1022,0.2875,0.0318</t>
-  </si>
-  <si>
-    <t>0.5527,0.1748,0.3296,0.0494</t>
-  </si>
-  <si>
-    <t>0.6367,0.1225,0.2743,0.0342</t>
-  </si>
-  <si>
-    <t>0.7432,0.0592,0.1976,0.0298</t>
-  </si>
-  <si>
-    <t>0.0731,0.0136,0.9601,0.0026</t>
-  </si>
-  <si>
-    <t>0.3317,0.0386,0.7539,0.0104</t>
-  </si>
-  <si>
-    <t>0.4491,0.0393,0.6286,0.0154</t>
-  </si>
-  <si>
-    <t>0.3585,0.0373,0.7138,0.0180</t>
-  </si>
-  <si>
-    <t>0.4605,0.2389,0.3864,0.0167</t>
-  </si>
-  <si>
-    <t>0.5681,0.1372,0.3410,0.0225</t>
-  </si>
-  <si>
-    <t>0.5027,0.2588,0.3140,0.0138</t>
-  </si>
-  <si>
-    <t>0.4877,0.1663,0.3994,0.0149</t>
-  </si>
-  <si>
-    <t>0.4935,0.2187,0.3812,0.0294</t>
-  </si>
-  <si>
-    <t>0.4620,0.2735,0.3502,0.0154</t>
-  </si>
-  <si>
-    <t>0.5117,0.2103,0.3631,0.0238</t>
-  </si>
-  <si>
-    <t>0.5555,0.0980,0.3857,0.0300</t>
-  </si>
-  <si>
-    <t>0.3052,0.0974,0.7065,0.0148</t>
-  </si>
-  <si>
-    <t>0.4787,0.0839,0.5018,0.0332</t>
-  </si>
-  <si>
-    <t>0.4934,0.0733,0.5358,0.0219</t>
-  </si>
-  <si>
-    <t>0.5212,0.1095,0.4194,0.0428</t>
-  </si>
-  <si>
-    <t>0.3936,0.3351,0.3360,0.0101</t>
-  </si>
-  <si>
-    <t>0.1006,0.7606,0.3651,0.0200</t>
-  </si>
-  <si>
-    <t>0.4669,0.1695,0.4670,0.0208</t>
-  </si>
-  <si>
-    <t>0.0744,0.7254,0.4940,0.0087</t>
-  </si>
-  <si>
-    <t>0.4896,0.1976,0.3720,0.0217</t>
-  </si>
-  <si>
-    <t>0.5382,0.1488,0.3509,0.0436</t>
-  </si>
-  <si>
-    <t>0.5081,0.2028,0.3510,0.0415</t>
-  </si>
-  <si>
-    <t>0.6014,0.1288,0.3384,0.0188</t>
-  </si>
-  <si>
-    <t>0.6127,0.1195,0.3056,0.0296</t>
-  </si>
-  <si>
-    <t>0.5450,0.1236,0.3715,0.0488</t>
-  </si>
-  <si>
-    <t>0.6910,0.0838,0.2474,0.0248</t>
-  </si>
-  <si>
-    <t>0.6100,0.1137,0.3477,0.0205</t>
-  </si>
-  <si>
-    <t>0.6470,0.0842,0.2880,0.0373</t>
-  </si>
-  <si>
-    <t>0.6406,0.1023,0.2817,0.0296</t>
-  </si>
-  <si>
-    <t>0.6908,0.0748,0.2602,0.0218</t>
-  </si>
-  <si>
-    <t>0.1871,0.1826,0.7184,0.0172</t>
-  </si>
-  <si>
-    <t>0.1228,0.2268,0.7797,0.0107</t>
-  </si>
-  <si>
-    <t>0.0983,0.1717,0.8252,0.0084</t>
-  </si>
-  <si>
-    <t>0.2914,0.0646,0.7279,0.0126</t>
-  </si>
-  <si>
-    <t>0.4620,0.0595,0.5251,0.0265</t>
-  </si>
-  <si>
-    <t>0.3544,0.1412,0.5119,0.0975</t>
-  </si>
-  <si>
-    <t>0.4635,0.0635,0.5293,0.0297</t>
-  </si>
-  <si>
-    <t>0.5617,0.0948,0.4081,0.0371</t>
-  </si>
-  <si>
-    <t>0.5920,0.0517,0.3195,0.0547</t>
-  </si>
-  <si>
-    <t>0.6376,0.0449,0.2858,0.0479</t>
-  </si>
-  <si>
-    <t>0.5125,0.0502,0.3610,0.0929</t>
-  </si>
-  <si>
-    <t>0.6147,0.0565,0.3030,0.0500</t>
-  </si>
-  <si>
-    <t>0.0854,0.3142,0.7784,0.0096</t>
-  </si>
-  <si>
-    <t>0.5759,0.1426,0.3195,0.0416</t>
-  </si>
-  <si>
-    <t>0.6132,0.1175,0.3298,0.0214</t>
-  </si>
-  <si>
-    <t>0.6267,0.0964,0.3226,0.0336</t>
-  </si>
-  <si>
-    <t>0.6505,0.1106,0.2631,0.0335</t>
-  </si>
-  <si>
-    <t>0.6263,0.0834,0.3416,0.0242</t>
-  </si>
-  <si>
-    <t>0.5248,0.0871,0.3689,0.0757</t>
-  </si>
-  <si>
-    <t>0.5716,0.1048,0.3637,0.0325</t>
-  </si>
-  <si>
-    <t>0.0466,0.1398,0.9082,0.0252</t>
-  </si>
-  <si>
-    <t>0.5978,0.0806,0.3293,0.0483</t>
-  </si>
-  <si>
-    <t>0.6003,0.1046,0.3013,0.0592</t>
-  </si>
-  <si>
-    <t>0.5132,0.0973,0.4762,0.0166</t>
-  </si>
-  <si>
-    <t>0.6402,0.0872,0.3178,0.0297</t>
-  </si>
-  <si>
-    <t>0.4972,0.1213,0.4701,0.0170</t>
-  </si>
-  <si>
-    <t>0.4710,0.1459,0.4548,0.0158</t>
-  </si>
-  <si>
-    <t>0.4947,0.1555,0.4040,0.0312</t>
-  </si>
-  <si>
-    <t>0.6269,0.0827,0.3121,0.0422</t>
-  </si>
-  <si>
-    <t>0.6129,0.0907,0.3300,0.0397</t>
-  </si>
-  <si>
-    <t>0.6169,0.1004,0.3011,0.0418</t>
-  </si>
-  <si>
-    <t>0.6310,0.1440,0.2464,0.0350</t>
-  </si>
-  <si>
-    <t>0.6023,0.1024,0.3511,0.0309</t>
-  </si>
-  <si>
-    <t>0.6475,0.1000,0.2994,0.0287</t>
-  </si>
-  <si>
-    <t>0.6257,0.0909,0.3507,0.0189</t>
-  </si>
-  <si>
-    <t>0.5570,0.1672,0.3603,0.0258</t>
-  </si>
-  <si>
-    <t>0.6188,0.1095,0.2684,0.0454</t>
-  </si>
-  <si>
-    <t>0.5313,0.1660,0.3637,0.0176</t>
-  </si>
-  <si>
-    <t>0.5081,0.2041,0.3707,0.0161</t>
-  </si>
-  <si>
-    <t>0.5722,0.1323,0.3369,0.0192</t>
-  </si>
-  <si>
-    <t>0.5970,0.1162,0.3371,0.0419</t>
-  </si>
-  <si>
-    <t>0.5669,0.1328,0.3849,0.0206</t>
-  </si>
-  <si>
-    <t>0.5464,0.1530,0.3096,0.0527</t>
-  </si>
-  <si>
-    <t>0.6329,0.1155,0.2561,0.0313</t>
-  </si>
-  <si>
-    <t>0.6858,0.0843,0.2259,0.0357</t>
-  </si>
-  <si>
-    <t>0.1912,0.0463,0.8448,0.0170</t>
-  </si>
-  <si>
-    <t>0.5508,0.1483,0.3257,0.0491</t>
-  </si>
-  <si>
-    <t>0.1442,0.0294,0.9019,0.0096</t>
-  </si>
-  <si>
-    <t>0.2145,0.0255,0.8537,0.0051</t>
-  </si>
-  <si>
-    <t>0.3314,0.0635,0.6989,0.0135</t>
-  </si>
-  <si>
-    <t>0.0694,0.2195,0.8582,0.0110</t>
-  </si>
-  <si>
-    <t>0.3172,0.1229,0.6435,0.0094</t>
-  </si>
-  <si>
-    <t>0.2964,0.0332,0.7644,0.0183</t>
-  </si>
-  <si>
-    <t>0.2587,0.0648,0.7769,0.0140</t>
-  </si>
-  <si>
-    <t>0.4692,0.0963,0.5363,0.0192</t>
-  </si>
-  <si>
-    <t>0.3844,0.0611,0.6609,0.0205</t>
-  </si>
-  <si>
-    <t>0.5158,0.0834,0.4967,0.0159</t>
-  </si>
-  <si>
-    <t>0.5078,0.1168,0.4874,0.0156</t>
-  </si>
-  <si>
-    <t>0.5017,0.1339,0.4373,0.0233</t>
-  </si>
-  <si>
-    <t>0.3511,0.1577,0.5527,0.0176</t>
-  </si>
-  <si>
-    <t>0.5438,0.1038,0.4500,0.0331</t>
-  </si>
-  <si>
-    <t>0.4994,0.0974,0.4506,0.0293</t>
-  </si>
-  <si>
-    <t>0.5688,0.1286,0.3631,0.0382</t>
-  </si>
-  <si>
-    <t>0.4412,0.1991,0.4617,0.0218</t>
-  </si>
-  <si>
-    <t>0.4637,0.1887,0.4326,0.0294</t>
-  </si>
-  <si>
-    <t>0.5983,0.1404,0.3325,0.0211</t>
-  </si>
-  <si>
-    <t>0.4630,0.2470,0.4253,0.0268</t>
-  </si>
-  <si>
-    <t>0.4614,0.1264,0.4998,0.0144</t>
-  </si>
-  <si>
-    <t>0.6203,0.0579,0.3894,0.0265</t>
-  </si>
-  <si>
-    <t>0.4809,0.1193,0.4723,0.0206</t>
-  </si>
-  <si>
-    <t>0.4768,0.0727,0.5407,0.0236</t>
-  </si>
-  <si>
-    <t>0.3698,0.0628,0.6758,0.0134</t>
-  </si>
-  <si>
-    <t>0.2901,0.0652,0.7306,0.0246</t>
-  </si>
-  <si>
-    <t>0.2685,0.0481,0.7818,0.0105</t>
-  </si>
-  <si>
-    <t>0.1828,0.0443,0.8614,0.0084</t>
-  </si>
-  <si>
-    <t>0.1493,0.0540,0.8582,0.0180</t>
-  </si>
-  <si>
-    <t>0.1293,0.2101,0.7742,0.0123</t>
-  </si>
-  <si>
-    <t>0.6823,0.0685,0.2372,0.0316</t>
-  </si>
-  <si>
-    <t>0.5880,0.1336,0.3157,0.0246</t>
-  </si>
-  <si>
-    <t>0.5816,0.1772,0.2921,0.0412</t>
-  </si>
-  <si>
-    <t>0.6414,0.1227,0.2577,0.0262</t>
-  </si>
-  <si>
-    <t>0.5881,0.1265,0.3241,0.0380</t>
-  </si>
-  <si>
-    <t>0.5553,0.1760,0.2975,0.0512</t>
-  </si>
-  <si>
-    <t>0.6833,0.0979,0.2355,0.0373</t>
-  </si>
-  <si>
-    <t>0.6697,0.1090,0.2508,0.0251</t>
-  </si>
-  <si>
-    <t>0.3672,0.0414,0.6936,0.0170</t>
-  </si>
-  <si>
-    <t>0.5081,0.0693,0.5022,0.0246</t>
-  </si>
-  <si>
-    <t>0.5173,0.1308,0.4031,0.0199</t>
-  </si>
-  <si>
-    <t>0.1115,0.0341,0.9069,0.0036</t>
-  </si>
-  <si>
-    <t>0.1085,0.1463,0.8249,0.0092</t>
-  </si>
-  <si>
-    <t>0.2790,0.1007,0.6889,0.0147</t>
-  </si>
-  <si>
-    <t>0.0334,0.0218,0.9735,0.0025</t>
-  </si>
-  <si>
-    <t>0.1605,0.0488,0.8529,0.0154</t>
-  </si>
-  <si>
-    <t>0.1520,0.0409,0.8789,0.0107</t>
-  </si>
-  <si>
-    <t>0.2092,0.1084,0.7614,0.0123</t>
-  </si>
-  <si>
-    <t>0.3965,0.0689,0.6344,0.0174</t>
-  </si>
-  <si>
-    <t>0.4299,0.0859,0.5733,0.0189</t>
-  </si>
-  <si>
-    <t>0.5474,0.0576,0.4656,0.0311</t>
-  </si>
-  <si>
-    <t>0.5317,0.0680,0.4911,0.0246</t>
-  </si>
-  <si>
-    <t>0.5701,0.1653,0.2841,0.0556</t>
-  </si>
-  <si>
-    <t>0.5999,0.1880,0.2642,0.0287</t>
-  </si>
-  <si>
-    <t>0.6521,0.1008,0.2983,0.0309</t>
-  </si>
-  <si>
-    <t>0.5922,0.1024,0.3734,0.0202</t>
-  </si>
-  <si>
-    <t>0.6483,0.1192,0.2337,0.0385</t>
-  </si>
-  <si>
-    <t>0.6633,0.1116,0.2142,0.0519</t>
-  </si>
-  <si>
-    <t>0.6466,0.1416,0.2411,0.0284</t>
-  </si>
-  <si>
-    <t>0.6285,0.1304,0.2344,0.0440</t>
-  </si>
-  <si>
-    <t>0.2003,0.1010,0.7603,0.0083</t>
-  </si>
-  <si>
-    <t>0.1401,0.1116,0.8075,0.0091</t>
-  </si>
-  <si>
-    <t>0.0509,0.0333,0.9523,0.0033</t>
-  </si>
-  <si>
-    <t>0.3888,0.1022,0.5910,0.0229</t>
-  </si>
-  <si>
-    <t>0.1268,0.0575,0.8835,0.0074</t>
-  </si>
-  <si>
-    <t>0.4486,0.0868,0.5144,0.0497</t>
-  </si>
-  <si>
-    <t>0.3735,0.0394,0.6967,0.0132</t>
-  </si>
-  <si>
-    <t>0.2605,0.0493,0.7463,0.0293</t>
-  </si>
-  <si>
-    <t>0.5327,0.1302,0.3791,0.0334</t>
-  </si>
-  <si>
-    <t>0.5882,0.0493,0.4132,0.0332</t>
-  </si>
-  <si>
-    <t>0.6858,0.0481,0.2528,0.0369</t>
-  </si>
-  <si>
-    <t>0.6045,0.0413,0.3255,0.0465</t>
-  </si>
-  <si>
-    <t>0.6403,0.0361,0.3084,0.0374</t>
-  </si>
-  <si>
-    <t>0.6173,0.0760,0.3245,0.0451</t>
+    <t>0.6023,0.0888,0.3513,0.0392</t>
+  </si>
+  <si>
+    <t>0.5476,0.0976,0.3682,0.0615</t>
+  </si>
+  <si>
+    <t>0.5501,0.1014,0.4076,0.0358</t>
+  </si>
+  <si>
+    <t>0.6246,0.0755,0.2936,0.0578</t>
+  </si>
+  <si>
+    <t>0.7182,0.0838,0.1645,0.0379</t>
+  </si>
+  <si>
+    <t>0.6913,0.0930,0.2381,0.0224</t>
+  </si>
+  <si>
+    <t>0.6169,0.1293,0.2591,0.0491</t>
+  </si>
+  <si>
+    <t>0.6356,0.0870,0.2815,0.0453</t>
+  </si>
+  <si>
+    <t>0.6297,0.1267,0.2615,0.0326</t>
+  </si>
+  <si>
+    <t>0.6071,0.1517,0.3009,0.0263</t>
+  </si>
+  <si>
+    <t>0.6020,0.1205,0.2921,0.0408</t>
+  </si>
+  <si>
+    <t>0.5345,0.2019,0.3498,0.0270</t>
+  </si>
+  <si>
+    <t>0.5663,0.0673,0.4792,0.0163</t>
+  </si>
+  <si>
+    <t>0.3422,0.1056,0.6434,0.0197</t>
+  </si>
+  <si>
+    <t>0.4521,0.0679,0.5820,0.0176</t>
+  </si>
+  <si>
+    <t>0.2905,0.0570,0.7503,0.0080</t>
+  </si>
+  <si>
+    <t>0.5207,0.0867,0.4780,0.0273</t>
+  </si>
+  <si>
+    <t>0.5491,0.2048,0.3181,0.0217</t>
+  </si>
+  <si>
+    <t>0.4254,0.2790,0.3746,0.0189</t>
+  </si>
+  <si>
+    <t>0.5989,0.1451,0.3098,0.0302</t>
+  </si>
+  <si>
+    <t>0.5018,0.2544,0.3307,0.0352</t>
+  </si>
+  <si>
+    <t>0.4531,0.2842,0.3646,0.0150</t>
+  </si>
+  <si>
+    <t>0.5851,0.0608,0.4498,0.0168</t>
+  </si>
+  <si>
+    <t>0.4939,0.0421,0.6165,0.0109</t>
+  </si>
+  <si>
+    <t>0.3357,0.0722,0.6737,0.0108</t>
+  </si>
+  <si>
+    <t>0.4306,0.0904,0.5815,0.0149</t>
+  </si>
+  <si>
+    <t>0.3809,0.1284,0.5753,0.0299</t>
+  </si>
+  <si>
+    <t>0.3626,0.1396,0.5899,0.0136</t>
+  </si>
+  <si>
+    <t>0.1365,0.0346,0.8970,0.0058</t>
+  </si>
+  <si>
+    <t>0.4961,0.1232,0.4417,0.0241</t>
+  </si>
+  <si>
+    <t>0.3685,0.1712,0.5746,0.0324</t>
+  </si>
+  <si>
+    <t>0.1096,0.0371,0.9203,0.0084</t>
+  </si>
+  <si>
+    <t>0.4347,0.1186,0.5474,0.0205</t>
+  </si>
+  <si>
+    <t>0.6165,0.1120,0.2891,0.0394</t>
+  </si>
+  <si>
+    <t>0.5124,0.1159,0.4420,0.0214</t>
+  </si>
+  <si>
+    <t>0.5806,0.1168,0.3654,0.0174</t>
+  </si>
+  <si>
+    <t>0.4494,0.2040,0.4451,0.0261</t>
+  </si>
+  <si>
+    <t>0.0908,0.3226,0.7223,0.0171</t>
+  </si>
+  <si>
+    <t>0.1140,0.0839,0.8620,0.0121</t>
+  </si>
+  <si>
+    <t>0.2724,0.0497,0.7529,0.0124</t>
+  </si>
+  <si>
+    <t>0.3726,0.0588,0.6628,0.0228</t>
+  </si>
+  <si>
+    <t>0.2595,0.0800,0.7398,0.0094</t>
+  </si>
+  <si>
+    <t>0.0700,0.4129,0.7203,0.0112</t>
+  </si>
+  <si>
+    <t>0.1835,0.1418,0.7453,0.0118</t>
+  </si>
+  <si>
+    <t>0.3052,0.1306,0.5302,0.1200</t>
+  </si>
+  <si>
+    <t>0.4278,0.2615,0.4024,0.0177</t>
+  </si>
+  <si>
+    <t>0.3227,0.3703,0.3899,0.0162</t>
+  </si>
+  <si>
+    <t>0.3446,0.4074,0.3988,0.0204</t>
+  </si>
+  <si>
+    <t>0.0448,0.2169,0.8773,0.0107</t>
+  </si>
+  <si>
+    <t>0.1296,0.0297,0.8999,0.0059</t>
+  </si>
+  <si>
+    <t>0.3246,0.0635,0.7020,0.0173</t>
+  </si>
+  <si>
+    <t>0.2983,0.0332,0.7685,0.0181</t>
+  </si>
+  <si>
+    <t>0.1637,0.0640,0.8405,0.0128</t>
+  </si>
+  <si>
+    <t>0.1526,0.0739,0.8495,0.0062</t>
+  </si>
+  <si>
+    <t>0.5629,0.2317,0.2741,0.0272</t>
+  </si>
+  <si>
+    <t>0.6549,0.0653,0.2812,0.0369</t>
+  </si>
+  <si>
+    <t>0.5619,0.1446,0.3313,0.0298</t>
+  </si>
+  <si>
+    <t>0.1186,0.0477,0.9032,0.0047</t>
+  </si>
+  <si>
+    <t>0.6649,0.1134,0.2545,0.0288</t>
+  </si>
+  <si>
+    <t>0.6769,0.0745,0.2664,0.0244</t>
+  </si>
+  <si>
+    <t>0.5958,0.1008,0.3712,0.0188</t>
+  </si>
+  <si>
+    <t>0.0877,0.1640,0.8576,0.0073</t>
+  </si>
+  <si>
+    <t>0.0242,0.2777,0.9151,0.0028</t>
+  </si>
+  <si>
+    <t>0.1056,0.2119,0.7600,0.0068</t>
+  </si>
+  <si>
+    <t>0.0570,0.5821,0.6318,0.0040</t>
+  </si>
+  <si>
+    <t>0.1445,0.0342,0.8874,0.0098</t>
+  </si>
+  <si>
+    <t>0.4321,0.2421,0.4515,0.0251</t>
+  </si>
+  <si>
+    <t>0.0302,0.9400,0.1396,0.0028</t>
+  </si>
+  <si>
+    <t>0.5885,0.1406,0.2610,0.0661</t>
+  </si>
+  <si>
+    <t>0.5601,0.1263,0.3225,0.0538</t>
+  </si>
+  <si>
+    <t>0.2230,0.0798,0.7836,0.0144</t>
+  </si>
+  <si>
+    <t>0.0672,0.3387,0.8214,0.0060</t>
+  </si>
+  <si>
+    <t>0.2157,0.2736,0.5803,0.0087</t>
+  </si>
+  <si>
+    <t>0.0150,0.9468,0.2321,0.0024</t>
+  </si>
+  <si>
+    <t>0.0234,0.1851,0.9364,0.0021</t>
+  </si>
+  <si>
+    <t>0.5114,0.0680,0.5228,0.0238</t>
+  </si>
+  <si>
+    <t>0.5400,0.0813,0.4217,0.0364</t>
+  </si>
+  <si>
+    <t>0.6069,0.0918,0.2629,0.0913</t>
+  </si>
+  <si>
+    <t>0.4964,0.0740,0.4215,0.0620</t>
+  </si>
+  <si>
+    <t>0.4682,0.0984,0.3878,0.0963</t>
+  </si>
+  <si>
+    <t>0.5207,0.0541,0.2767,0.1253</t>
+  </si>
+  <si>
+    <t>0.0532,0.2269,0.8687,0.0051</t>
+  </si>
+  <si>
+    <t>0.0210,0.6115,0.8040,0.0033</t>
+  </si>
+  <si>
+    <t>0.0827,0.3442,0.7681,0.0109</t>
+  </si>
+  <si>
+    <t>0.1000,0.1573,0.8360,0.0064</t>
+  </si>
+  <si>
+    <t>0.1724,0.1443,0.7613,0.0093</t>
+  </si>
+  <si>
+    <t>0.2074,0.1196,0.7280,0.0048</t>
+  </si>
+  <si>
+    <t>0.6660,0.1103,0.2435,0.0328</t>
+  </si>
+  <si>
+    <t>0.6977,0.1036,0.1947,0.0354</t>
+  </si>
+  <si>
+    <t>0.5548,0.1417,0.3266,0.0366</t>
+  </si>
+  <si>
+    <t>0.6277,0.1235,0.2766,0.0365</t>
+  </si>
+  <si>
+    <t>0.6042,0.1175,0.3098,0.0241</t>
+  </si>
+  <si>
+    <t>0.5818,0.1774,0.2686,0.0473</t>
+  </si>
+  <si>
+    <t>0.5717,0.1260,0.3644,0.0214</t>
+  </si>
+  <si>
+    <t>0.6708,0.1000,0.2498,0.0355</t>
+  </si>
+  <si>
+    <t>0.6325,0.1236,0.2407,0.0376</t>
+  </si>
+  <si>
+    <t>0.5833,0.1348,0.3556,0.0243</t>
+  </si>
+  <si>
+    <t>0.5342,0.2012,0.3389,0.0350</t>
+  </si>
+  <si>
+    <t>0.5995,0.1342,0.3070,0.0471</t>
+  </si>
+  <si>
+    <t>0.6385,0.0982,0.3001,0.0315</t>
+  </si>
+  <si>
+    <t>0.6147,0.0923,0.3527,0.0315</t>
+  </si>
+  <si>
+    <t>0.6524,0.0929,0.2647,0.0335</t>
+  </si>
+  <si>
+    <t>0.5982,0.1794,0.2538,0.0413</t>
+  </si>
+  <si>
+    <t>0.1278,0.0409,0.9000,0.0057</t>
+  </si>
+  <si>
+    <t>0.4725,0.0817,0.5087,0.0189</t>
+  </si>
+  <si>
+    <t>0.4816,0.0774,0.5112,0.0191</t>
+  </si>
+  <si>
+    <t>0.4128,0.0918,0.5587,0.0161</t>
+  </si>
+  <si>
+    <t>0.4332,0.2892,0.3732,0.0273</t>
+  </si>
+  <si>
+    <t>0.4385,0.2613,0.3554,0.0104</t>
+  </si>
+  <si>
+    <t>0.3979,0.3720,0.3502,0.0185</t>
+  </si>
+  <si>
+    <t>0.5349,0.1950,0.3514,0.0179</t>
+  </si>
+  <si>
+    <t>0.5713,0.1817,0.2999,0.0205</t>
+  </si>
+  <si>
+    <t>0.3257,0.4691,0.2989,0.0111</t>
+  </si>
+  <si>
+    <t>0.3744,0.2807,0.4271,0.0143</t>
+  </si>
+  <si>
+    <t>0.5001,0.1230,0.4534,0.0329</t>
+  </si>
+  <si>
+    <t>0.4036,0.0520,0.6668,0.0152</t>
+  </si>
+  <si>
+    <t>0.5502,0.0621,0.4027,0.0405</t>
+  </si>
+  <si>
+    <t>0.4582,0.0703,0.5612,0.0205</t>
+  </si>
+  <si>
+    <t>0.5605,0.0894,0.3909,0.0367</t>
+  </si>
+  <si>
+    <t>0.3084,0.4256,0.3256,0.0091</t>
+  </si>
+  <si>
+    <t>0.4040,0.2344,0.4689,0.0169</t>
+  </si>
+  <si>
+    <t>0.5142,0.1184,0.4256,0.0246</t>
+  </si>
+  <si>
+    <t>0.0826,0.7799,0.2941,0.0054</t>
+  </si>
+  <si>
+    <t>0.5097,0.2000,0.3708,0.0226</t>
+  </si>
+  <si>
+    <t>0.6317,0.1340,0.2194,0.0606</t>
+  </si>
+  <si>
+    <t>0.7107,0.0830,0.2014,0.0249</t>
+  </si>
+  <si>
+    <t>0.6139,0.1193,0.3303,0.0236</t>
+  </si>
+  <si>
+    <t>0.6770,0.0819,0.2066,0.0495</t>
+  </si>
+  <si>
+    <t>0.5981,0.1402,0.3097,0.0304</t>
+  </si>
+  <si>
+    <t>0.6195,0.1290,0.2985,0.0279</t>
+  </si>
+  <si>
+    <t>0.6170,0.1009,0.3235,0.0317</t>
+  </si>
+  <si>
+    <t>0.5022,0.2086,0.3928,0.0215</t>
+  </si>
+  <si>
+    <t>0.5989,0.0903,0.3355,0.0299</t>
+  </si>
+  <si>
+    <t>0.6030,0.1287,0.3042,0.0373</t>
+  </si>
+  <si>
+    <t>0.1526,0.1269,0.7985,0.0111</t>
+  </si>
+  <si>
+    <t>0.2163,0.1837,0.6522,0.0066</t>
+  </si>
+  <si>
+    <t>0.0929,0.1065,0.8756,0.0055</t>
+  </si>
+  <si>
+    <t>0.2378,0.0405,0.8294,0.0072</t>
+  </si>
+  <si>
+    <t>0.5305,0.0629,0.4408,0.0320</t>
+  </si>
+  <si>
+    <t>0.3870,0.0656,0.6305,0.0285</t>
+  </si>
+  <si>
+    <t>0.4928,0.0676,0.5311,0.0177</t>
+  </si>
+  <si>
+    <t>0.5855,0.0509,0.4298,0.0199</t>
+  </si>
+  <si>
+    <t>0.6465,0.0535,0.2147,0.0663</t>
+  </si>
+  <si>
+    <t>0.4861,0.0743,0.4403,0.0585</t>
+  </si>
+  <si>
+    <t>0.5690,0.0533,0.3517,0.0594</t>
+  </si>
+  <si>
+    <t>0.6214,0.0443,0.3551,0.0289</t>
+  </si>
+  <si>
+    <t>0.0140,0.6651,0.8188,0.0034</t>
+  </si>
+  <si>
+    <t>0.5382,0.1695,0.3743,0.0304</t>
+  </si>
+  <si>
+    <t>0.5848,0.1116,0.3587,0.0222</t>
+  </si>
+  <si>
+    <t>0.6241,0.1112,0.2729,0.0434</t>
+  </si>
+  <si>
+    <t>0.5143,0.2286,0.3366,0.0254</t>
+  </si>
+  <si>
+    <t>0.6270,0.1118,0.3053,0.0273</t>
+  </si>
+  <si>
+    <t>0.4666,0.1578,0.3852,0.0791</t>
+  </si>
+  <si>
+    <t>0.6006,0.1292,0.3058,0.0470</t>
+  </si>
+  <si>
+    <t>0.0453,0.0770,0.9261,0.0279</t>
+  </si>
+  <si>
+    <t>0.6310,0.0944,0.2633,0.0514</t>
+  </si>
+  <si>
+    <t>0.5906,0.0897,0.2870,0.0783</t>
+  </si>
+  <si>
+    <t>0.5222,0.1501,0.4209,0.0179</t>
+  </si>
+  <si>
+    <t>0.5869,0.0836,0.3870,0.0233</t>
+  </si>
+  <si>
+    <t>0.5992,0.1082,0.3273,0.0422</t>
+  </si>
+  <si>
+    <t>0.4565,0.1547,0.4810,0.0389</t>
+  </si>
+  <si>
+    <t>0.5647,0.0966,0.4276,0.0295</t>
+  </si>
+  <si>
+    <t>0.5478,0.1163,0.4077,0.0324</t>
+  </si>
+  <si>
+    <t>0.5797,0.1249,0.3544,0.0280</t>
+  </si>
+  <si>
+    <t>0.5928,0.1231,0.2841,0.0448</t>
+  </si>
+  <si>
+    <t>0.6600,0.0624,0.2758,0.0362</t>
+  </si>
+  <si>
+    <t>0.6732,0.0824,0.1853,0.0574</t>
+  </si>
+  <si>
+    <t>0.6218,0.0793,0.3832,0.0207</t>
+  </si>
+  <si>
+    <t>0.5603,0.1769,0.3271,0.0347</t>
+  </si>
+  <si>
+    <t>0.6230,0.0982,0.3445,0.0204</t>
+  </si>
+  <si>
+    <t>0.5852,0.1191,0.3218,0.0417</t>
+  </si>
+  <si>
+    <t>0.6640,0.1072,0.2398,0.0258</t>
+  </si>
+  <si>
+    <t>0.4857,0.2148,0.3449,0.0221</t>
+  </si>
+  <si>
+    <t>0.5945,0.1347,0.3006,0.0258</t>
+  </si>
+  <si>
+    <t>0.6208,0.0920,0.3211,0.0260</t>
+  </si>
+  <si>
+    <t>0.6095,0.1609,0.2831,0.0268</t>
+  </si>
+  <si>
+    <t>0.6519,0.1125,0.2757,0.0213</t>
+  </si>
+  <si>
+    <t>0.5515,0.1770,0.3481,0.0294</t>
+  </si>
+  <si>
+    <t>0.5837,0.1287,0.3507,0.0187</t>
+  </si>
+  <si>
+    <t>0.3039,0.0593,0.7337,0.0083</t>
+  </si>
+  <si>
+    <t>0.6083,0.1130,0.3478,0.0166</t>
+  </si>
+  <si>
+    <t>0.1629,0.0813,0.8363,0.0145</t>
+  </si>
+  <si>
+    <t>0.2600,0.0726,0.7480,0.0168</t>
+  </si>
+  <si>
+    <t>0.3450,0.0689,0.6792,0.0158</t>
+  </si>
+  <si>
+    <t>0.0664,0.0895,0.9211,0.0075</t>
+  </si>
+  <si>
+    <t>0.3174,0.0742,0.7056,0.0143</t>
+  </si>
+  <si>
+    <t>0.2285,0.0527,0.8005,0.0068</t>
+  </si>
+  <si>
+    <t>0.1751,0.0755,0.8386,0.0117</t>
+  </si>
+  <si>
+    <t>0.4116,0.1117,0.5783,0.0285</t>
+  </si>
+  <si>
+    <t>0.4539,0.0781,0.5624,0.0166</t>
+  </si>
+  <si>
+    <t>0.4449,0.0691,0.5883,0.0152</t>
+  </si>
+  <si>
+    <t>0.4127,0.1143,0.5845,0.0251</t>
+  </si>
+  <si>
+    <t>0.4743,0.1037,0.5273,0.0201</t>
+  </si>
+  <si>
+    <t>0.3635,0.1479,0.5772,0.0077</t>
+  </si>
+  <si>
+    <t>0.5215,0.0654,0.4804,0.0192</t>
+  </si>
+  <si>
+    <t>0.4810,0.1058,0.4773,0.0307</t>
+  </si>
+  <si>
+    <t>0.5328,0.1640,0.3616,0.0277</t>
+  </si>
+  <si>
+    <t>0.6196,0.1239,0.3052,0.0260</t>
+  </si>
+  <si>
+    <t>0.5718,0.1359,0.3441,0.0245</t>
+  </si>
+  <si>
+    <t>0.6249,0.1043,0.3159,0.0278</t>
+  </si>
+  <si>
+    <t>0.6083,0.1687,0.2759,0.0261</t>
+  </si>
+  <si>
+    <t>0.5133,0.0665,0.5010,0.0259</t>
+  </si>
+  <si>
+    <t>0.4787,0.0929,0.5139,0.0198</t>
+  </si>
+  <si>
+    <t>0.4777,0.1065,0.4706,0.0366</t>
+  </si>
+  <si>
+    <t>0.3745,0.0885,0.6371,0.0151</t>
+  </si>
+  <si>
+    <t>0.4413,0.1124,0.5114,0.0218</t>
+  </si>
+  <si>
+    <t>0.1251,0.1013,0.8622,0.0059</t>
+  </si>
+  <si>
+    <t>0.2516,0.0529,0.7870,0.0147</t>
+  </si>
+  <si>
+    <t>0.2474,0.0676,0.7623,0.0224</t>
+  </si>
+  <si>
+    <t>0.1104,0.0533,0.8957,0.0049</t>
+  </si>
+  <si>
+    <t>0.1034,0.2206,0.7865,0.0086</t>
+  </si>
+  <si>
+    <t>0.6112,0.1286,0.2469,0.0481</t>
+  </si>
+  <si>
+    <t>0.5888,0.1510,0.2801,0.0382</t>
+  </si>
+  <si>
+    <t>0.5769,0.1430,0.2829,0.0446</t>
+  </si>
+  <si>
+    <t>0.5529,0.1771,0.3436,0.0286</t>
+  </si>
+  <si>
+    <t>0.6332,0.0832,0.3211,0.0305</t>
+  </si>
+  <si>
+    <t>0.6026,0.1846,0.2587,0.0292</t>
+  </si>
+  <si>
+    <t>0.6353,0.1644,0.2481,0.0239</t>
+  </si>
+  <si>
+    <t>0.5890,0.1456,0.3198,0.0240</t>
+  </si>
+  <si>
+    <t>0.4527,0.1028,0.5499,0.0157</t>
+  </si>
+  <si>
+    <t>0.5198,0.1391,0.4061,0.0284</t>
+  </si>
+  <si>
+    <t>0.5313,0.1035,0.4205,0.0247</t>
+  </si>
+  <si>
+    <t>0.1651,0.0742,0.8355,0.0095</t>
+  </si>
+  <si>
+    <t>0.1883,0.0595,0.8126,0.0106</t>
+  </si>
+  <si>
+    <t>0.3302,0.0710,0.6755,0.0144</t>
+  </si>
+  <si>
+    <t>0.0653,0.0281,0.9510,0.0041</t>
+  </si>
+  <si>
+    <t>0.2557,0.0821,0.7598,0.0185</t>
+  </si>
+  <si>
+    <t>0.0449,0.0180,0.9641,0.0038</t>
+  </si>
+  <si>
+    <t>0.1379,0.0798,0.8464,0.0057</t>
+  </si>
+  <si>
+    <t>0.3551,0.0670,0.6741,0.0115</t>
+  </si>
+  <si>
+    <t>0.3761,0.1059,0.5796,0.0393</t>
+  </si>
+  <si>
+    <t>0.5512,0.0790,0.4178,0.0259</t>
+  </si>
+  <si>
+    <t>0.6110,0.0605,0.3609,0.0331</t>
+  </si>
+  <si>
+    <t>0.7163,0.0724,0.2340,0.0250</t>
+  </si>
+  <si>
+    <t>0.6229,0.1284,0.2767,0.0387</t>
+  </si>
+  <si>
+    <t>0.6708,0.0843,0.2447,0.0320</t>
+  </si>
+  <si>
+    <t>0.6176,0.1190,0.2958,0.0325</t>
+  </si>
+  <si>
+    <t>0.5961,0.1990,0.2326,0.0452</t>
+  </si>
+  <si>
+    <t>0.6264,0.1158,0.2427,0.0530</t>
+  </si>
+  <si>
+    <t>0.6648,0.1069,0.2241,0.0388</t>
+  </si>
+  <si>
+    <t>0.5863,0.1656,0.2856,0.0440</t>
+  </si>
+  <si>
+    <t>0.2310,0.0666,0.7909,0.0107</t>
+  </si>
+  <si>
+    <t>0.0776,0.1135,0.8980,0.0055</t>
+  </si>
+  <si>
+    <t>0.1701,0.1423,0.7833,0.0090</t>
+  </si>
+  <si>
+    <t>0.3015,0.1614,0.6329,0.0196</t>
+  </si>
+  <si>
+    <t>0.2408,0.0612,0.7811,0.0131</t>
+  </si>
+  <si>
+    <t>0.4973,0.0476,0.5552,0.0132</t>
+  </si>
+  <si>
+    <t>0.5750,0.0386,0.4651,0.0187</t>
+  </si>
+  <si>
+    <t>0.2708,0.0599,0.7415,0.0245</t>
+  </si>
+  <si>
+    <t>0.5677,0.0808,0.3469,0.0516</t>
+  </si>
+  <si>
+    <t>0.4864,0.0423,0.3849,0.0882</t>
+  </si>
+  <si>
+    <t>0.6534,0.0532,0.2987,0.0353</t>
+  </si>
+  <si>
+    <t>0.5947,0.0535,0.3009,0.0745</t>
+  </si>
+  <si>
+    <t>0.5683,0.0631,0.2893,0.0922</t>
+  </si>
+  <si>
+    <t>0.5483,0.0636,0.4337,0.0272</t>
   </si>
 </sst>
 </file>
@@ -1953,7 +1953,7 @@
         <v>259</v>
       </c>
       <c r="C2" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D2" t="s">
         <v>264</v>
@@ -2121,7 +2121,7 @@
         <v>259</v>
       </c>
       <c r="C14" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D14" t="s">
         <v>276</v>
@@ -2135,7 +2135,7 @@
         <v>261</v>
       </c>
       <c r="C15" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D15" t="s">
         <v>277</v>
@@ -2261,7 +2261,7 @@
         <v>259</v>
       </c>
       <c r="C24" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D24" t="s">
         <v>286</v>
@@ -2373,7 +2373,7 @@
         <v>259</v>
       </c>
       <c r="C32" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D32" t="s">
         <v>294</v>
@@ -2541,7 +2541,7 @@
         <v>262</v>
       </c>
       <c r="C44" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D44" t="s">
         <v>306</v>
@@ -2569,7 +2569,7 @@
         <v>259</v>
       </c>
       <c r="C46" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D46" t="s">
         <v>308</v>
@@ -2849,7 +2849,7 @@
         <v>263</v>
       </c>
       <c r="C66" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D66" t="s">
         <v>328</v>
@@ -2975,7 +2975,7 @@
         <v>262</v>
       </c>
       <c r="C75" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D75" t="s">
         <v>337</v>
@@ -3003,7 +3003,7 @@
         <v>260</v>
       </c>
       <c r="C77" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D77" t="s">
         <v>339</v>
@@ -3087,7 +3087,7 @@
         <v>263</v>
       </c>
       <c r="C83" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D83" t="s">
         <v>345</v>
@@ -3101,7 +3101,7 @@
         <v>261</v>
       </c>
       <c r="C84" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D84" t="s">
         <v>346</v>
@@ -3143,7 +3143,7 @@
         <v>263</v>
       </c>
       <c r="C87" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D87" t="s">
         <v>349</v>
@@ -3577,7 +3577,7 @@
         <v>259</v>
       </c>
       <c r="C118" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D118" t="s">
         <v>380</v>
@@ -3633,7 +3633,7 @@
         <v>262</v>
       </c>
       <c r="C122" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D122" t="s">
         <v>384</v>
@@ -3885,7 +3885,7 @@
         <v>259</v>
       </c>
       <c r="C140" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D140" t="s">
         <v>402</v>
@@ -3997,7 +3997,7 @@
         <v>263</v>
       </c>
       <c r="C148" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D148" t="s">
         <v>410</v>
@@ -4613,7 +4613,7 @@
         <v>259</v>
       </c>
       <c r="C192" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D192" t="s">
         <v>454</v>
@@ -4627,7 +4627,7 @@
         <v>261</v>
       </c>
       <c r="C193" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D193" t="s">
         <v>455</v>
@@ -4641,7 +4641,7 @@
         <v>261</v>
       </c>
       <c r="C194" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D194" t="s">
         <v>456</v>
@@ -4767,7 +4767,7 @@
         <v>259</v>
       </c>
       <c r="C203" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D203" t="s">
         <v>465</v>
@@ -4781,7 +4781,7 @@
         <v>259</v>
       </c>
       <c r="C204" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D204" t="s">
         <v>466</v>
@@ -5033,7 +5033,7 @@
         <v>259</v>
       </c>
       <c r="C222" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D222" t="s">
         <v>484</v>
@@ -5411,7 +5411,7 @@
         <v>261</v>
       </c>
       <c r="C249" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D249" t="s">
         <v>511</v>

</xml_diff>

<commit_message>
add new clasify runs fr average metrics
</commit_message>
<xml_diff>
--- a/dataset_agreed/saved_models/hyperparameter_optimized_runs/pointcloud_HPO_run_1/epoch_10/per_file_predictions_epoch_10.xlsx
+++ b/dataset_agreed/saved_models/hyperparameter_optimized_runs/pointcloud_HPO_run_1/epoch_10/per_file_predictions_epoch_10.xlsx
@@ -808,769 +808,769 @@
     <t>0,1,1,0</t>
   </si>
   <si>
-    <t>0.6023,0.0888,0.3513,0.0392</t>
-  </si>
-  <si>
-    <t>0.5476,0.0976,0.3682,0.0615</t>
-  </si>
-  <si>
-    <t>0.5501,0.1014,0.4076,0.0358</t>
-  </si>
-  <si>
-    <t>0.6246,0.0755,0.2936,0.0578</t>
-  </si>
-  <si>
-    <t>0.7182,0.0838,0.1645,0.0379</t>
-  </si>
-  <si>
-    <t>0.6913,0.0930,0.2381,0.0224</t>
-  </si>
-  <si>
-    <t>0.6169,0.1293,0.2591,0.0491</t>
-  </si>
-  <si>
-    <t>0.6356,0.0870,0.2815,0.0453</t>
-  </si>
-  <si>
-    <t>0.6297,0.1267,0.2615,0.0326</t>
-  </si>
-  <si>
-    <t>0.6071,0.1517,0.3009,0.0263</t>
-  </si>
-  <si>
-    <t>0.6020,0.1205,0.2921,0.0408</t>
-  </si>
-  <si>
-    <t>0.5345,0.2019,0.3498,0.0270</t>
-  </si>
-  <si>
-    <t>0.5663,0.0673,0.4792,0.0163</t>
-  </si>
-  <si>
-    <t>0.3422,0.1056,0.6434,0.0197</t>
-  </si>
-  <si>
-    <t>0.4521,0.0679,0.5820,0.0176</t>
-  </si>
-  <si>
-    <t>0.2905,0.0570,0.7503,0.0080</t>
-  </si>
-  <si>
-    <t>0.5207,0.0867,0.4780,0.0273</t>
-  </si>
-  <si>
-    <t>0.5491,0.2048,0.3181,0.0217</t>
-  </si>
-  <si>
-    <t>0.4254,0.2790,0.3746,0.0189</t>
-  </si>
-  <si>
-    <t>0.5989,0.1451,0.3098,0.0302</t>
-  </si>
-  <si>
-    <t>0.5018,0.2544,0.3307,0.0352</t>
-  </si>
-  <si>
-    <t>0.4531,0.2842,0.3646,0.0150</t>
-  </si>
-  <si>
-    <t>0.5851,0.0608,0.4498,0.0168</t>
-  </si>
-  <si>
-    <t>0.4939,0.0421,0.6165,0.0109</t>
-  </si>
-  <si>
-    <t>0.3357,0.0722,0.6737,0.0108</t>
-  </si>
-  <si>
-    <t>0.4306,0.0904,0.5815,0.0149</t>
-  </si>
-  <si>
-    <t>0.3809,0.1284,0.5753,0.0299</t>
-  </si>
-  <si>
-    <t>0.3626,0.1396,0.5899,0.0136</t>
-  </si>
-  <si>
-    <t>0.1365,0.0346,0.8970,0.0058</t>
-  </si>
-  <si>
-    <t>0.4961,0.1232,0.4417,0.0241</t>
-  </si>
-  <si>
-    <t>0.3685,0.1712,0.5746,0.0324</t>
-  </si>
-  <si>
-    <t>0.1096,0.0371,0.9203,0.0084</t>
-  </si>
-  <si>
-    <t>0.4347,0.1186,0.5474,0.0205</t>
-  </si>
-  <si>
-    <t>0.6165,0.1120,0.2891,0.0394</t>
-  </si>
-  <si>
-    <t>0.5124,0.1159,0.4420,0.0214</t>
-  </si>
-  <si>
-    <t>0.5806,0.1168,0.3654,0.0174</t>
-  </si>
-  <si>
-    <t>0.4494,0.2040,0.4451,0.0261</t>
-  </si>
-  <si>
-    <t>0.0908,0.3226,0.7223,0.0171</t>
-  </si>
-  <si>
-    <t>0.1140,0.0839,0.8620,0.0121</t>
-  </si>
-  <si>
-    <t>0.2724,0.0497,0.7529,0.0124</t>
-  </si>
-  <si>
-    <t>0.3726,0.0588,0.6628,0.0228</t>
-  </si>
-  <si>
-    <t>0.2595,0.0800,0.7398,0.0094</t>
-  </si>
-  <si>
-    <t>0.0700,0.4129,0.7203,0.0112</t>
-  </si>
-  <si>
-    <t>0.1835,0.1418,0.7453,0.0118</t>
-  </si>
-  <si>
-    <t>0.3052,0.1306,0.5302,0.1200</t>
-  </si>
-  <si>
-    <t>0.4278,0.2615,0.4024,0.0177</t>
-  </si>
-  <si>
-    <t>0.3227,0.3703,0.3899,0.0162</t>
-  </si>
-  <si>
-    <t>0.3446,0.4074,0.3988,0.0204</t>
-  </si>
-  <si>
-    <t>0.0448,0.2169,0.8773,0.0107</t>
-  </si>
-  <si>
-    <t>0.1296,0.0297,0.8999,0.0059</t>
-  </si>
-  <si>
-    <t>0.3246,0.0635,0.7020,0.0173</t>
-  </si>
-  <si>
-    <t>0.2983,0.0332,0.7685,0.0181</t>
-  </si>
-  <si>
-    <t>0.1637,0.0640,0.8405,0.0128</t>
-  </si>
-  <si>
-    <t>0.1526,0.0739,0.8495,0.0062</t>
-  </si>
-  <si>
-    <t>0.5629,0.2317,0.2741,0.0272</t>
-  </si>
-  <si>
-    <t>0.6549,0.0653,0.2812,0.0369</t>
-  </si>
-  <si>
-    <t>0.5619,0.1446,0.3313,0.0298</t>
-  </si>
-  <si>
-    <t>0.1186,0.0477,0.9032,0.0047</t>
-  </si>
-  <si>
-    <t>0.6649,0.1134,0.2545,0.0288</t>
-  </si>
-  <si>
-    <t>0.6769,0.0745,0.2664,0.0244</t>
-  </si>
-  <si>
-    <t>0.5958,0.1008,0.3712,0.0188</t>
-  </si>
-  <si>
-    <t>0.0877,0.1640,0.8576,0.0073</t>
-  </si>
-  <si>
-    <t>0.0242,0.2777,0.9151,0.0028</t>
-  </si>
-  <si>
-    <t>0.1056,0.2119,0.7600,0.0068</t>
-  </si>
-  <si>
-    <t>0.0570,0.5821,0.6318,0.0040</t>
-  </si>
-  <si>
-    <t>0.1445,0.0342,0.8874,0.0098</t>
-  </si>
-  <si>
-    <t>0.4321,0.2421,0.4515,0.0251</t>
-  </si>
-  <si>
-    <t>0.0302,0.9400,0.1396,0.0028</t>
-  </si>
-  <si>
-    <t>0.5885,0.1406,0.2610,0.0661</t>
-  </si>
-  <si>
-    <t>0.5601,0.1263,0.3225,0.0538</t>
-  </si>
-  <si>
-    <t>0.2230,0.0798,0.7836,0.0144</t>
-  </si>
-  <si>
-    <t>0.0672,0.3387,0.8214,0.0060</t>
-  </si>
-  <si>
-    <t>0.2157,0.2736,0.5803,0.0087</t>
-  </si>
-  <si>
-    <t>0.0150,0.9468,0.2321,0.0024</t>
-  </si>
-  <si>
-    <t>0.0234,0.1851,0.9364,0.0021</t>
-  </si>
-  <si>
-    <t>0.5114,0.0680,0.5228,0.0238</t>
-  </si>
-  <si>
-    <t>0.5400,0.0813,0.4217,0.0364</t>
-  </si>
-  <si>
-    <t>0.6069,0.0918,0.2629,0.0913</t>
-  </si>
-  <si>
-    <t>0.4964,0.0740,0.4215,0.0620</t>
-  </si>
-  <si>
-    <t>0.4682,0.0984,0.3878,0.0963</t>
-  </si>
-  <si>
-    <t>0.5207,0.0541,0.2767,0.1253</t>
-  </si>
-  <si>
-    <t>0.0532,0.2269,0.8687,0.0051</t>
-  </si>
-  <si>
-    <t>0.0210,0.6115,0.8040,0.0033</t>
-  </si>
-  <si>
-    <t>0.0827,0.3442,0.7681,0.0109</t>
-  </si>
-  <si>
-    <t>0.1000,0.1573,0.8360,0.0064</t>
-  </si>
-  <si>
-    <t>0.1724,0.1443,0.7613,0.0093</t>
-  </si>
-  <si>
-    <t>0.2074,0.1196,0.7280,0.0048</t>
-  </si>
-  <si>
-    <t>0.6660,0.1103,0.2435,0.0328</t>
-  </si>
-  <si>
-    <t>0.6977,0.1036,0.1947,0.0354</t>
-  </si>
-  <si>
-    <t>0.5548,0.1417,0.3266,0.0366</t>
-  </si>
-  <si>
-    <t>0.6277,0.1235,0.2766,0.0365</t>
-  </si>
-  <si>
-    <t>0.6042,0.1175,0.3098,0.0241</t>
-  </si>
-  <si>
-    <t>0.5818,0.1774,0.2686,0.0473</t>
-  </si>
-  <si>
-    <t>0.5717,0.1260,0.3644,0.0214</t>
-  </si>
-  <si>
-    <t>0.6708,0.1000,0.2498,0.0355</t>
-  </si>
-  <si>
-    <t>0.6325,0.1236,0.2407,0.0376</t>
-  </si>
-  <si>
-    <t>0.5833,0.1348,0.3556,0.0243</t>
-  </si>
-  <si>
-    <t>0.5342,0.2012,0.3389,0.0350</t>
-  </si>
-  <si>
-    <t>0.5995,0.1342,0.3070,0.0471</t>
-  </si>
-  <si>
-    <t>0.6385,0.0982,0.3001,0.0315</t>
-  </si>
-  <si>
-    <t>0.6147,0.0923,0.3527,0.0315</t>
-  </si>
-  <si>
-    <t>0.6524,0.0929,0.2647,0.0335</t>
-  </si>
-  <si>
-    <t>0.5982,0.1794,0.2538,0.0413</t>
-  </si>
-  <si>
-    <t>0.1278,0.0409,0.9000,0.0057</t>
-  </si>
-  <si>
-    <t>0.4725,0.0817,0.5087,0.0189</t>
-  </si>
-  <si>
-    <t>0.4816,0.0774,0.5112,0.0191</t>
-  </si>
-  <si>
-    <t>0.4128,0.0918,0.5587,0.0161</t>
-  </si>
-  <si>
-    <t>0.4332,0.2892,0.3732,0.0273</t>
-  </si>
-  <si>
-    <t>0.4385,0.2613,0.3554,0.0104</t>
-  </si>
-  <si>
-    <t>0.3979,0.3720,0.3502,0.0185</t>
-  </si>
-  <si>
-    <t>0.5349,0.1950,0.3514,0.0179</t>
-  </si>
-  <si>
-    <t>0.5713,0.1817,0.2999,0.0205</t>
-  </si>
-  <si>
-    <t>0.3257,0.4691,0.2989,0.0111</t>
-  </si>
-  <si>
-    <t>0.3744,0.2807,0.4271,0.0143</t>
-  </si>
-  <si>
-    <t>0.5001,0.1230,0.4534,0.0329</t>
-  </si>
-  <si>
-    <t>0.4036,0.0520,0.6668,0.0152</t>
-  </si>
-  <si>
-    <t>0.5502,0.0621,0.4027,0.0405</t>
-  </si>
-  <si>
-    <t>0.4582,0.0703,0.5612,0.0205</t>
-  </si>
-  <si>
-    <t>0.5605,0.0894,0.3909,0.0367</t>
-  </si>
-  <si>
-    <t>0.3084,0.4256,0.3256,0.0091</t>
-  </si>
-  <si>
-    <t>0.4040,0.2344,0.4689,0.0169</t>
-  </si>
-  <si>
-    <t>0.5142,0.1184,0.4256,0.0246</t>
-  </si>
-  <si>
-    <t>0.0826,0.7799,0.2941,0.0054</t>
-  </si>
-  <si>
-    <t>0.5097,0.2000,0.3708,0.0226</t>
-  </si>
-  <si>
-    <t>0.6317,0.1340,0.2194,0.0606</t>
-  </si>
-  <si>
-    <t>0.7107,0.0830,0.2014,0.0249</t>
-  </si>
-  <si>
-    <t>0.6139,0.1193,0.3303,0.0236</t>
-  </si>
-  <si>
-    <t>0.6770,0.0819,0.2066,0.0495</t>
-  </si>
-  <si>
-    <t>0.5981,0.1402,0.3097,0.0304</t>
-  </si>
-  <si>
-    <t>0.6195,0.1290,0.2985,0.0279</t>
-  </si>
-  <si>
-    <t>0.6170,0.1009,0.3235,0.0317</t>
-  </si>
-  <si>
-    <t>0.5022,0.2086,0.3928,0.0215</t>
-  </si>
-  <si>
-    <t>0.5989,0.0903,0.3355,0.0299</t>
-  </si>
-  <si>
-    <t>0.6030,0.1287,0.3042,0.0373</t>
-  </si>
-  <si>
-    <t>0.1526,0.1269,0.7985,0.0111</t>
-  </si>
-  <si>
-    <t>0.2163,0.1837,0.6522,0.0066</t>
-  </si>
-  <si>
-    <t>0.0929,0.1065,0.8756,0.0055</t>
-  </si>
-  <si>
-    <t>0.2378,0.0405,0.8294,0.0072</t>
-  </si>
-  <si>
-    <t>0.5305,0.0629,0.4408,0.0320</t>
-  </si>
-  <si>
-    <t>0.3870,0.0656,0.6305,0.0285</t>
-  </si>
-  <si>
-    <t>0.4928,0.0676,0.5311,0.0177</t>
-  </si>
-  <si>
-    <t>0.5855,0.0509,0.4298,0.0199</t>
-  </si>
-  <si>
-    <t>0.6465,0.0535,0.2147,0.0663</t>
-  </si>
-  <si>
-    <t>0.4861,0.0743,0.4403,0.0585</t>
-  </si>
-  <si>
-    <t>0.5690,0.0533,0.3517,0.0594</t>
-  </si>
-  <si>
-    <t>0.6214,0.0443,0.3551,0.0289</t>
-  </si>
-  <si>
-    <t>0.0140,0.6651,0.8188,0.0034</t>
-  </si>
-  <si>
-    <t>0.5382,0.1695,0.3743,0.0304</t>
-  </si>
-  <si>
-    <t>0.5848,0.1116,0.3587,0.0222</t>
-  </si>
-  <si>
-    <t>0.6241,0.1112,0.2729,0.0434</t>
-  </si>
-  <si>
-    <t>0.5143,0.2286,0.3366,0.0254</t>
-  </si>
-  <si>
-    <t>0.6270,0.1118,0.3053,0.0273</t>
-  </si>
-  <si>
-    <t>0.4666,0.1578,0.3852,0.0791</t>
-  </si>
-  <si>
-    <t>0.6006,0.1292,0.3058,0.0470</t>
-  </si>
-  <si>
-    <t>0.0453,0.0770,0.9261,0.0279</t>
-  </si>
-  <si>
-    <t>0.6310,0.0944,0.2633,0.0514</t>
-  </si>
-  <si>
-    <t>0.5906,0.0897,0.2870,0.0783</t>
-  </si>
-  <si>
-    <t>0.5222,0.1501,0.4209,0.0179</t>
-  </si>
-  <si>
-    <t>0.5869,0.0836,0.3870,0.0233</t>
-  </si>
-  <si>
-    <t>0.5992,0.1082,0.3273,0.0422</t>
-  </si>
-  <si>
-    <t>0.4565,0.1547,0.4810,0.0389</t>
-  </si>
-  <si>
-    <t>0.5647,0.0966,0.4276,0.0295</t>
-  </si>
-  <si>
-    <t>0.5478,0.1163,0.4077,0.0324</t>
-  </si>
-  <si>
-    <t>0.5797,0.1249,0.3544,0.0280</t>
-  </si>
-  <si>
-    <t>0.5928,0.1231,0.2841,0.0448</t>
-  </si>
-  <si>
-    <t>0.6600,0.0624,0.2758,0.0362</t>
-  </si>
-  <si>
-    <t>0.6732,0.0824,0.1853,0.0574</t>
-  </si>
-  <si>
-    <t>0.6218,0.0793,0.3832,0.0207</t>
-  </si>
-  <si>
-    <t>0.5603,0.1769,0.3271,0.0347</t>
-  </si>
-  <si>
-    <t>0.6230,0.0982,0.3445,0.0204</t>
-  </si>
-  <si>
-    <t>0.5852,0.1191,0.3218,0.0417</t>
-  </si>
-  <si>
-    <t>0.6640,0.1072,0.2398,0.0258</t>
-  </si>
-  <si>
-    <t>0.4857,0.2148,0.3449,0.0221</t>
-  </si>
-  <si>
-    <t>0.5945,0.1347,0.3006,0.0258</t>
-  </si>
-  <si>
-    <t>0.6208,0.0920,0.3211,0.0260</t>
-  </si>
-  <si>
-    <t>0.6095,0.1609,0.2831,0.0268</t>
-  </si>
-  <si>
-    <t>0.6519,0.1125,0.2757,0.0213</t>
-  </si>
-  <si>
-    <t>0.5515,0.1770,0.3481,0.0294</t>
-  </si>
-  <si>
-    <t>0.5837,0.1287,0.3507,0.0187</t>
-  </si>
-  <si>
-    <t>0.3039,0.0593,0.7337,0.0083</t>
-  </si>
-  <si>
-    <t>0.6083,0.1130,0.3478,0.0166</t>
-  </si>
-  <si>
-    <t>0.1629,0.0813,0.8363,0.0145</t>
-  </si>
-  <si>
-    <t>0.2600,0.0726,0.7480,0.0168</t>
-  </si>
-  <si>
-    <t>0.3450,0.0689,0.6792,0.0158</t>
-  </si>
-  <si>
-    <t>0.0664,0.0895,0.9211,0.0075</t>
-  </si>
-  <si>
-    <t>0.3174,0.0742,0.7056,0.0143</t>
-  </si>
-  <si>
-    <t>0.2285,0.0527,0.8005,0.0068</t>
-  </si>
-  <si>
-    <t>0.1751,0.0755,0.8386,0.0117</t>
-  </si>
-  <si>
-    <t>0.4116,0.1117,0.5783,0.0285</t>
-  </si>
-  <si>
-    <t>0.4539,0.0781,0.5624,0.0166</t>
-  </si>
-  <si>
-    <t>0.4449,0.0691,0.5883,0.0152</t>
-  </si>
-  <si>
-    <t>0.4127,0.1143,0.5845,0.0251</t>
-  </si>
-  <si>
-    <t>0.4743,0.1037,0.5273,0.0201</t>
-  </si>
-  <si>
-    <t>0.3635,0.1479,0.5772,0.0077</t>
-  </si>
-  <si>
-    <t>0.5215,0.0654,0.4804,0.0192</t>
-  </si>
-  <si>
-    <t>0.4810,0.1058,0.4773,0.0307</t>
-  </si>
-  <si>
-    <t>0.5328,0.1640,0.3616,0.0277</t>
-  </si>
-  <si>
-    <t>0.6196,0.1239,0.3052,0.0260</t>
-  </si>
-  <si>
-    <t>0.5718,0.1359,0.3441,0.0245</t>
-  </si>
-  <si>
-    <t>0.6249,0.1043,0.3159,0.0278</t>
-  </si>
-  <si>
-    <t>0.6083,0.1687,0.2759,0.0261</t>
-  </si>
-  <si>
-    <t>0.5133,0.0665,0.5010,0.0259</t>
-  </si>
-  <si>
-    <t>0.4787,0.0929,0.5139,0.0198</t>
-  </si>
-  <si>
-    <t>0.4777,0.1065,0.4706,0.0366</t>
-  </si>
-  <si>
-    <t>0.3745,0.0885,0.6371,0.0151</t>
-  </si>
-  <si>
-    <t>0.4413,0.1124,0.5114,0.0218</t>
-  </si>
-  <si>
-    <t>0.1251,0.1013,0.8622,0.0059</t>
-  </si>
-  <si>
-    <t>0.2516,0.0529,0.7870,0.0147</t>
-  </si>
-  <si>
-    <t>0.2474,0.0676,0.7623,0.0224</t>
-  </si>
-  <si>
-    <t>0.1104,0.0533,0.8957,0.0049</t>
-  </si>
-  <si>
-    <t>0.1034,0.2206,0.7865,0.0086</t>
-  </si>
-  <si>
-    <t>0.6112,0.1286,0.2469,0.0481</t>
-  </si>
-  <si>
-    <t>0.5888,0.1510,0.2801,0.0382</t>
-  </si>
-  <si>
-    <t>0.5769,0.1430,0.2829,0.0446</t>
-  </si>
-  <si>
-    <t>0.5529,0.1771,0.3436,0.0286</t>
-  </si>
-  <si>
-    <t>0.6332,0.0832,0.3211,0.0305</t>
-  </si>
-  <si>
-    <t>0.6026,0.1846,0.2587,0.0292</t>
-  </si>
-  <si>
-    <t>0.6353,0.1644,0.2481,0.0239</t>
-  </si>
-  <si>
-    <t>0.5890,0.1456,0.3198,0.0240</t>
-  </si>
-  <si>
-    <t>0.4527,0.1028,0.5499,0.0157</t>
-  </si>
-  <si>
-    <t>0.5198,0.1391,0.4061,0.0284</t>
-  </si>
-  <si>
-    <t>0.5313,0.1035,0.4205,0.0247</t>
-  </si>
-  <si>
-    <t>0.1651,0.0742,0.8355,0.0095</t>
-  </si>
-  <si>
-    <t>0.1883,0.0595,0.8126,0.0106</t>
-  </si>
-  <si>
-    <t>0.3302,0.0710,0.6755,0.0144</t>
-  </si>
-  <si>
-    <t>0.0653,0.0281,0.9510,0.0041</t>
-  </si>
-  <si>
-    <t>0.2557,0.0821,0.7598,0.0185</t>
-  </si>
-  <si>
-    <t>0.0449,0.0180,0.9641,0.0038</t>
-  </si>
-  <si>
-    <t>0.1379,0.0798,0.8464,0.0057</t>
-  </si>
-  <si>
-    <t>0.3551,0.0670,0.6741,0.0115</t>
-  </si>
-  <si>
-    <t>0.3761,0.1059,0.5796,0.0393</t>
-  </si>
-  <si>
-    <t>0.5512,0.0790,0.4178,0.0259</t>
-  </si>
-  <si>
-    <t>0.6110,0.0605,0.3609,0.0331</t>
-  </si>
-  <si>
-    <t>0.7163,0.0724,0.2340,0.0250</t>
-  </si>
-  <si>
-    <t>0.6229,0.1284,0.2767,0.0387</t>
-  </si>
-  <si>
-    <t>0.6708,0.0843,0.2447,0.0320</t>
-  </si>
-  <si>
-    <t>0.6176,0.1190,0.2958,0.0325</t>
-  </si>
-  <si>
-    <t>0.5961,0.1990,0.2326,0.0452</t>
-  </si>
-  <si>
-    <t>0.6264,0.1158,0.2427,0.0530</t>
-  </si>
-  <si>
-    <t>0.6648,0.1069,0.2241,0.0388</t>
-  </si>
-  <si>
-    <t>0.5863,0.1656,0.2856,0.0440</t>
-  </si>
-  <si>
-    <t>0.2310,0.0666,0.7909,0.0107</t>
-  </si>
-  <si>
-    <t>0.0776,0.1135,0.8980,0.0055</t>
-  </si>
-  <si>
-    <t>0.1701,0.1423,0.7833,0.0090</t>
-  </si>
-  <si>
-    <t>0.3015,0.1614,0.6329,0.0196</t>
-  </si>
-  <si>
-    <t>0.2408,0.0612,0.7811,0.0131</t>
-  </si>
-  <si>
-    <t>0.4973,0.0476,0.5552,0.0132</t>
-  </si>
-  <si>
-    <t>0.5750,0.0386,0.4651,0.0187</t>
-  </si>
-  <si>
-    <t>0.2708,0.0599,0.7415,0.0245</t>
-  </si>
-  <si>
-    <t>0.5677,0.0808,0.3469,0.0516</t>
-  </si>
-  <si>
-    <t>0.4864,0.0423,0.3849,0.0882</t>
-  </si>
-  <si>
-    <t>0.6534,0.0532,0.2987,0.0353</t>
-  </si>
-  <si>
-    <t>0.5947,0.0535,0.3009,0.0745</t>
-  </si>
-  <si>
-    <t>0.5683,0.0631,0.2893,0.0922</t>
-  </si>
-  <si>
-    <t>0.5483,0.0636,0.4337,0.0272</t>
+    <t>0.5793,0.0416,0.0312,0.4618</t>
+  </si>
+  <si>
+    <t>0.0383,0.0083,0.0041,0.9812</t>
+  </si>
+  <si>
+    <t>0.7920,0.0198,0.0259,0.1745</t>
+  </si>
+  <si>
+    <t>0.3482,0.0197,0.2385,0.3632</t>
+  </si>
+  <si>
+    <t>0.9792,0.0194,0.0016,0.0027</t>
+  </si>
+  <si>
+    <t>0.9768,0.0194,0.0023,0.0032</t>
+  </si>
+  <si>
+    <t>0.9559,0.0544,0.0031,0.0029</t>
+  </si>
+  <si>
+    <t>0.9749,0.0177,0.0012,0.0062</t>
+  </si>
+  <si>
+    <t>0.9515,0.0622,0.0026,0.0034</t>
+  </si>
+  <si>
+    <t>0.9320,0.0863,0.0033,0.0056</t>
+  </si>
+  <si>
+    <t>0.9556,0.0638,0.0023,0.0022</t>
+  </si>
+  <si>
+    <t>0.9788,0.0172,0.0015,0.0052</t>
+  </si>
+  <si>
+    <t>0.5929,0.1073,0.3785,0.0188</t>
+  </si>
+  <si>
+    <t>0.2034,0.0231,0.8666,0.0036</t>
+  </si>
+  <si>
+    <t>0.0815,0.0183,0.9481,0.0048</t>
+  </si>
+  <si>
+    <t>0.0459,0.0104,0.9776,0.0015</t>
+  </si>
+  <si>
+    <t>0.5703,0.0628,0.4539,0.0279</t>
+  </si>
+  <si>
+    <t>0.0404,0.9526,0.0278,0.0028</t>
+  </si>
+  <si>
+    <t>0.0211,0.9802,0.0108,0.0015</t>
+  </si>
+  <si>
+    <t>0.1801,0.8584,0.0161,0.0044</t>
+  </si>
+  <si>
+    <t>0.0264,0.9737,0.0070,0.0018</t>
+  </si>
+  <si>
+    <t>0.0090,0.9887,0.0045,0.0008</t>
+  </si>
+  <si>
+    <t>0.4387,0.0135,0.7174,0.0107</t>
+  </si>
+  <si>
+    <t>0.1837,0.0195,0.8634,0.0200</t>
+  </si>
+  <si>
+    <t>0.0064,0.0036,0.9961,0.0006</t>
+  </si>
+  <si>
+    <t>0.1179,0.0147,0.9327,0.0052</t>
+  </si>
+  <si>
+    <t>0.0600,0.0088,0.9700,0.0031</t>
+  </si>
+  <si>
+    <t>0.0610,0.0061,0.9740,0.0017</t>
+  </si>
+  <si>
+    <t>0.0064,0.0036,0.9956,0.0013</t>
+  </si>
+  <si>
+    <t>0.1695,0.7681,0.1356,0.0114</t>
+  </si>
+  <si>
+    <t>0.3819,0.0718,0.6526,0.0153</t>
+  </si>
+  <si>
+    <t>0.0014,0.0032,0.9989,0.0004</t>
+  </si>
+  <si>
+    <t>0.0534,0.2004,0.8644,0.0024</t>
+  </si>
+  <si>
+    <t>0.5708,0.1364,0.3225,0.0106</t>
+  </si>
+  <si>
+    <t>0.4347,0.1645,0.4823,0.0266</t>
+  </si>
+  <si>
+    <t>0.4126,0.6495,0.0206,0.0043</t>
+  </si>
+  <si>
+    <t>0.0926,0.8305,0.3052,0.0079</t>
+  </si>
+  <si>
+    <t>0.0093,0.2821,0.9480,0.0038</t>
+  </si>
+  <si>
+    <t>0.0324,0.0240,0.9674,0.0041</t>
+  </si>
+  <si>
+    <t>0.0211,0.0740,0.9644,0.0028</t>
+  </si>
+  <si>
+    <t>0.0581,0.0053,0.9712,0.0046</t>
+  </si>
+  <si>
+    <t>0.0202,0.0225,0.9822,0.0010</t>
+  </si>
+  <si>
+    <t>0.0177,0.9284,0.1121,0.0021</t>
+  </si>
+  <si>
+    <t>0.0615,0.0226,0.9509,0.0036</t>
+  </si>
+  <si>
+    <t>0.3008,0.3680,0.1731,0.5024</t>
+  </si>
+  <si>
+    <t>0.0266,0.9433,0.1283,0.0040</t>
+  </si>
+  <si>
+    <t>0.0079,0.9751,0.1988,0.0011</t>
+  </si>
+  <si>
+    <t>0.0204,0.9609,0.0993,0.0035</t>
+  </si>
+  <si>
+    <t>0.0036,0.3035,0.9695,0.0015</t>
+  </si>
+  <si>
+    <t>0.0033,0.0211,0.9951,0.0005</t>
+  </si>
+  <si>
+    <t>0.0360,0.0038,0.9850,0.0022</t>
+  </si>
+  <si>
+    <t>0.0250,0.0030,0.9875,0.0031</t>
+  </si>
+  <si>
+    <t>0.0062,0.0174,0.9923,0.0017</t>
+  </si>
+  <si>
+    <t>0.0172,0.0241,0.9830,0.0020</t>
+  </si>
+  <si>
+    <t>0.9480,0.0711,0.0025,0.0038</t>
+  </si>
+  <si>
+    <t>0.8595,0.1705,0.0106,0.0053</t>
+  </si>
+  <si>
+    <t>0.7876,0.2894,0.0083,0.0035</t>
+  </si>
+  <si>
+    <t>0.0189,0.1952,0.9491,0.0029</t>
+  </si>
+  <si>
+    <t>0.9625,0.0303,0.0056,0.0045</t>
+  </si>
+  <si>
+    <t>0.8773,0.1870,0.0044,0.0036</t>
+  </si>
+  <si>
+    <t>0.6359,0.4873,0.0072,0.0055</t>
+  </si>
+  <si>
+    <t>0.0010,0.7011,0.9647,0.0005</t>
+  </si>
+  <si>
+    <t>0.0033,0.0235,0.9946,0.0005</t>
+  </si>
+  <si>
+    <t>0.0037,0.0512,0.9914,0.0012</t>
+  </si>
+  <si>
+    <t>0.0022,0.6834,0.9449,0.0007</t>
+  </si>
+  <si>
+    <t>0.0019,0.0103,0.9973,0.0005</t>
+  </si>
+  <si>
+    <t>0.0682,0.6753,0.5796,0.0049</t>
+  </si>
+  <si>
+    <t>0.0146,0.9777,0.0231,0.0009</t>
+  </si>
+  <si>
+    <t>0.6748,0.0361,0.2451,0.0686</t>
+  </si>
+  <si>
+    <t>0.4733,0.1255,0.4862,0.0139</t>
+  </si>
+  <si>
+    <t>0.0130,0.0934,0.9692,0.0024</t>
+  </si>
+  <si>
+    <t>0.0011,0.9193,0.8860,0.0003</t>
+  </si>
+  <si>
+    <t>0.0044,0.8167,0.8720,0.0008</t>
+  </si>
+  <si>
+    <t>0.0031,0.9018,0.7842,0.0013</t>
+  </si>
+  <si>
+    <t>0.0020,0.9177,0.8505,0.0010</t>
+  </si>
+  <si>
+    <t>0.0318,0.0258,0.0997,0.9325</t>
+  </si>
+  <si>
+    <t>0.0314,0.0255,0.0165,0.9709</t>
+  </si>
+  <si>
+    <t>0.0241,0.0274,0.0138,0.9773</t>
+  </si>
+  <si>
+    <t>0.0680,0.0469,0.0501,0.9298</t>
+  </si>
+  <si>
+    <t>0.1369,0.0716,0.0589,0.8729</t>
+  </si>
+  <si>
+    <t>0.0349,0.0149,0.0407,0.9555</t>
+  </si>
+  <si>
+    <t>0.0015,0.8756,0.9041,0.0005</t>
+  </si>
+  <si>
+    <t>0.0090,0.5549,0.9000,0.0035</t>
+  </si>
+  <si>
+    <t>0.0061,0.5293,0.9295,0.0020</t>
+  </si>
+  <si>
+    <t>0.0078,0.2982,0.9559,0.0013</t>
+  </si>
+  <si>
+    <t>0.0038,0.7126,0.9117,0.0011</t>
+  </si>
+  <si>
+    <t>0.0069,0.7815,0.8384,0.0019</t>
+  </si>
+  <si>
+    <t>0.8885,0.1240,0.0064,0.0084</t>
+  </si>
+  <si>
+    <t>0.9049,0.1268,0.0032,0.0050</t>
+  </si>
+  <si>
+    <t>0.9119,0.1174,0.0038,0.0045</t>
+  </si>
+  <si>
+    <t>0.9494,0.0349,0.0019,0.0111</t>
+  </si>
+  <si>
+    <t>0.9723,0.0245,0.0023,0.0048</t>
+  </si>
+  <si>
+    <t>0.8412,0.2599,0.0032,0.0023</t>
+  </si>
+  <si>
+    <t>0.8236,0.2299,0.0103,0.0038</t>
+  </si>
+  <si>
+    <t>0.8599,0.1657,0.0059,0.0100</t>
+  </si>
+  <si>
+    <t>0.9846,0.0088,0.0008,0.0064</t>
+  </si>
+  <si>
+    <t>0.9833,0.0140,0.0009,0.0029</t>
+  </si>
+  <si>
+    <t>0.9842,0.0106,0.0009,0.0042</t>
+  </si>
+  <si>
+    <t>0.9898,0.0070,0.0008,0.0023</t>
+  </si>
+  <si>
+    <t>0.9761,0.0240,0.0013,0.0031</t>
+  </si>
+  <si>
+    <t>0.9817,0.0155,0.0013,0.0028</t>
+  </si>
+  <si>
+    <t>0.9656,0.0356,0.0014,0.0048</t>
+  </si>
+  <si>
+    <t>0.9846,0.0124,0.0013,0.0030</t>
+  </si>
+  <si>
+    <t>0.0045,0.0037,0.9967,0.0008</t>
+  </si>
+  <si>
+    <t>0.0203,0.0096,0.9872,0.0016</t>
+  </si>
+  <si>
+    <t>0.5351,0.0337,0.4267,0.0715</t>
+  </si>
+  <si>
+    <t>0.1171,0.0121,0.9369,0.0051</t>
+  </si>
+  <si>
+    <t>0.0815,0.9254,0.0190,0.0027</t>
+  </si>
+  <si>
+    <t>0.0781,0.9307,0.0125,0.0027</t>
+  </si>
+  <si>
+    <t>0.0862,0.9306,0.0061,0.0014</t>
+  </si>
+  <si>
+    <t>0.1028,0.9123,0.0084,0.0025</t>
+  </si>
+  <si>
+    <t>0.0270,0.9681,0.0198,0.0024</t>
+  </si>
+  <si>
+    <t>0.0183,0.9797,0.0062,0.0021</t>
+  </si>
+  <si>
+    <t>0.1706,0.8645,0.0186,0.0038</t>
+  </si>
+  <si>
+    <t>0.5926,0.0877,0.3721,0.0170</t>
+  </si>
+  <si>
+    <t>0.1260,0.0118,0.9356,0.0046</t>
+  </si>
+  <si>
+    <t>0.2803,0.0645,0.7558,0.0246</t>
+  </si>
+  <si>
+    <t>0.4137,0.0226,0.7535,0.0068</t>
+  </si>
+  <si>
+    <t>0.5048,0.0913,0.5152,0.0570</t>
+  </si>
+  <si>
+    <t>0.0104,0.9798,0.0697,0.0017</t>
+  </si>
+  <si>
+    <t>0.0120,0.9747,0.0852,0.0028</t>
+  </si>
+  <si>
+    <t>0.1960,0.6188,0.3020,0.0163</t>
+  </si>
+  <si>
+    <t>0.0008,0.9880,0.5347,0.0004</t>
+  </si>
+  <si>
+    <t>0.0967,0.8584,0.1099,0.0020</t>
+  </si>
+  <si>
+    <t>0.5847,0.4732,0.0227,0.0037</t>
+  </si>
+  <si>
+    <t>0.2789,0.7645,0.0173,0.0033</t>
+  </si>
+  <si>
+    <t>0.9573,0.0399,0.0050,0.0047</t>
+  </si>
+  <si>
+    <t>0.9539,0.0249,0.0042,0.0202</t>
+  </si>
+  <si>
+    <t>0.9807,0.0113,0.0027,0.0053</t>
+  </si>
+  <si>
+    <t>0.9125,0.0800,0.0135,0.0065</t>
+  </si>
+  <si>
+    <t>0.9573,0.0214,0.0029,0.0216</t>
+  </si>
+  <si>
+    <t>0.8940,0.1121,0.0138,0.0067</t>
+  </si>
+  <si>
+    <t>0.9406,0.0551,0.0073,0.0067</t>
+  </si>
+  <si>
+    <t>0.9680,0.0264,0.0033,0.0054</t>
+  </si>
+  <si>
+    <t>0.0033,0.1134,0.9878,0.0003</t>
+  </si>
+  <si>
+    <t>0.0101,0.2737,0.9491,0.0008</t>
+  </si>
+  <si>
+    <t>0.0139,0.0507,0.9799,0.0008</t>
+  </si>
+  <si>
+    <t>0.0185,0.0124,0.9876,0.0008</t>
+  </si>
+  <si>
+    <t>0.4965,0.0363,0.6154,0.0173</t>
+  </si>
+  <si>
+    <t>0.5664,0.0603,0.4596,0.0493</t>
+  </si>
+  <si>
+    <t>0.1664,0.0040,0.9491,0.0016</t>
+  </si>
+  <si>
+    <t>0.5237,0.0499,0.5723,0.0102</t>
+  </si>
+  <si>
+    <t>0.0121,0.0121,0.0228,0.9824</t>
+  </si>
+  <si>
+    <t>0.0089,0.0048,0.0226,0.9847</t>
+  </si>
+  <si>
+    <t>0.0246,0.0194,0.0498,0.9602</t>
+  </si>
+  <si>
+    <t>0.0441,0.0128,0.0114,0.9685</t>
+  </si>
+  <si>
+    <t>0.0015,0.9104,0.8738,0.0012</t>
+  </si>
+  <si>
+    <t>0.9629,0.0223,0.0059,0.0125</t>
+  </si>
+  <si>
+    <t>0.2772,0.7306,0.0222,0.0133</t>
+  </si>
+  <si>
+    <t>0.8714,0.1344,0.0108,0.0280</t>
+  </si>
+  <si>
+    <t>0.6632,0.3757,0.0289,0.0084</t>
+  </si>
+  <si>
+    <t>0.9607,0.0168,0.0100,0.0144</t>
+  </si>
+  <si>
+    <t>0.5789,0.0387,0.2659,0.1225</t>
+  </si>
+  <si>
+    <t>0.9440,0.0288,0.0065,0.0239</t>
+  </si>
+  <si>
+    <t>0.0039,0.1055,0.9825,0.0041</t>
+  </si>
+  <si>
+    <t>0.5948,0.0126,0.0268,0.4697</t>
+  </si>
+  <si>
+    <t>0.8813,0.0090,0.0159,0.0921</t>
+  </si>
+  <si>
+    <t>0.5136,0.1828,0.3587,0.0158</t>
+  </si>
+  <si>
+    <t>0.5628,0.1585,0.2952,0.0195</t>
+  </si>
+  <si>
+    <t>0.6942,0.1263,0.2075,0.0283</t>
+  </si>
+  <si>
+    <t>0.3659,0.2373,0.4706,0.0157</t>
+  </si>
+  <si>
+    <t>0.3167,0.2487,0.4401,0.0115</t>
+  </si>
+  <si>
+    <t>0.5532,0.1850,0.3012,0.0145</t>
+  </si>
+  <si>
+    <t>0.9308,0.0572,0.0109,0.0071</t>
+  </si>
+  <si>
+    <t>0.9773,0.0125,0.0015,0.0083</t>
+  </si>
+  <si>
+    <t>0.9707,0.0166,0.0033,0.0086</t>
+  </si>
+  <si>
+    <t>0.9721,0.0142,0.0033,0.0110</t>
+  </si>
+  <si>
+    <t>0.9798,0.0132,0.0022,0.0055</t>
+  </si>
+  <si>
+    <t>0.9622,0.0281,0.0047,0.0078</t>
+  </si>
+  <si>
+    <t>0.9013,0.1182,0.0089,0.0062</t>
+  </si>
+  <si>
+    <t>0.9842,0.0076,0.0016,0.0058</t>
+  </si>
+  <si>
+    <t>0.2710,0.7865,0.0161,0.0041</t>
+  </si>
+  <si>
+    <t>0.5069,0.5882,0.0121,0.0029</t>
+  </si>
+  <si>
+    <t>0.1779,0.8282,0.0273,0.0029</t>
+  </si>
+  <si>
+    <t>0.6668,0.1247,0.2386,0.0151</t>
+  </si>
+  <si>
+    <t>0.8665,0.1683,0.0065,0.0044</t>
+  </si>
+  <si>
+    <t>0.8777,0.1287,0.0138,0.0065</t>
+  </si>
+  <si>
+    <t>0.8527,0.1695,0.0081,0.0061</t>
+  </si>
+  <si>
+    <t>0.8543,0.1050,0.0175,0.0358</t>
+  </si>
+  <si>
+    <t>0.0020,0.0085,0.9978,0.0004</t>
+  </si>
+  <si>
+    <t>0.8019,0.2147,0.0197,0.0058</t>
+  </si>
+  <si>
+    <t>0.0049,0.0128,0.9937,0.0013</t>
+  </si>
+  <si>
+    <t>0.0127,0.0644,0.9784,0.0017</t>
+  </si>
+  <si>
+    <t>0.0676,0.0121,0.9686,0.0013</t>
+  </si>
+  <si>
+    <t>0.0060,0.0506,0.9873,0.0016</t>
+  </si>
+  <si>
+    <t>0.0187,0.0057,0.9898,0.0010</t>
+  </si>
+  <si>
+    <t>0.0168,0.0061,0.9897,0.0013</t>
+  </si>
+  <si>
+    <t>0.0031,0.0036,0.9976,0.0005</t>
+  </si>
+  <si>
+    <t>0.1907,0.0187,0.8919,0.0067</t>
+  </si>
+  <si>
+    <t>0.1755,0.0115,0.9055,0.0086</t>
+  </si>
+  <si>
+    <t>0.0797,0.0645,0.9183,0.0042</t>
+  </si>
+  <si>
+    <t>0.3668,0.0555,0.6767,0.0051</t>
+  </si>
+  <si>
+    <t>0.3211,0.1015,0.6465,0.0080</t>
+  </si>
+  <si>
+    <t>0.3573,0.0457,0.7394,0.0125</t>
+  </si>
+  <si>
+    <t>0.3073,0.5012,0.3569,0.0934</t>
+  </si>
+  <si>
+    <t>0.3978,0.0317,0.7226,0.0061</t>
+  </si>
+  <si>
+    <t>0.1669,0.8718,0.0062,0.0033</t>
+  </si>
+  <si>
+    <t>0.1555,0.8802,0.0053,0.0020</t>
+  </si>
+  <si>
+    <t>0.1015,0.9055,0.0154,0.0024</t>
+  </si>
+  <si>
+    <t>0.7695,0.3115,0.0111,0.0053</t>
+  </si>
+  <si>
+    <t>0.2903,0.7827,0.0061,0.0032</t>
+  </si>
+  <si>
+    <t>0.4339,0.0878,0.5317,0.0165</t>
+  </si>
+  <si>
+    <t>0.5397,0.0151,0.6146,0.0115</t>
+  </si>
+  <si>
+    <t>0.4828,0.0233,0.6393,0.0151</t>
+  </si>
+  <si>
+    <t>0.4410,0.0139,0.7522,0.0068</t>
+  </si>
+  <si>
+    <t>0.3141,0.0349,0.7533,0.0158</t>
+  </si>
+  <si>
+    <t>0.0445,0.0161,0.9641,0.0102</t>
+  </si>
+  <si>
+    <t>0.0370,0.0740,0.9491,0.0046</t>
+  </si>
+  <si>
+    <t>0.0603,0.0744,0.9236,0.0039</t>
+  </si>
+  <si>
+    <t>0.0086,0.0222,0.9897,0.0007</t>
+  </si>
+  <si>
+    <t>0.0056,0.3528,0.9528,0.0026</t>
+  </si>
+  <si>
+    <t>0.9587,0.0412,0.0025,0.0058</t>
+  </si>
+  <si>
+    <t>0.9438,0.0743,0.0038,0.0027</t>
+  </si>
+  <si>
+    <t>0.9517,0.0494,0.0024,0.0056</t>
+  </si>
+  <si>
+    <t>0.9367,0.0671,0.0052,0.0071</t>
+  </si>
+  <si>
+    <t>0.9205,0.1010,0.0046,0.0047</t>
+  </si>
+  <si>
+    <t>0.9144,0.1168,0.0039,0.0055</t>
+  </si>
+  <si>
+    <t>0.9665,0.0353,0.0016,0.0046</t>
+  </si>
+  <si>
+    <t>0.9564,0.0402,0.0020,0.0067</t>
+  </si>
+  <si>
+    <t>0.0807,0.0101,0.9679,0.0016</t>
+  </si>
+  <si>
+    <t>0.2509,0.3011,0.5865,0.0077</t>
+  </si>
+  <si>
+    <t>0.5486,0.1017,0.3692,0.0157</t>
+  </si>
+  <si>
+    <t>0.0037,0.0041,0.9972,0.0004</t>
+  </si>
+  <si>
+    <t>0.0013,0.0121,0.9974,0.0006</t>
+  </si>
+  <si>
+    <t>0.0245,0.0092,0.9850,0.0015</t>
+  </si>
+  <si>
+    <t>0.0030,0.0052,0.9975,0.0003</t>
+  </si>
+  <si>
+    <t>0.0434,0.0270,0.9650,0.0026</t>
+  </si>
+  <si>
+    <t>0.0042,0.0393,0.9913,0.0017</t>
+  </si>
+  <si>
+    <t>0.0065,0.0060,0.9943,0.0012</t>
+  </si>
+  <si>
+    <t>0.2339,0.0400,0.8341,0.0072</t>
+  </si>
+  <si>
+    <t>0.4238,0.0191,0.6846,0.0176</t>
+  </si>
+  <si>
+    <t>0.6442,0.0149,0.4698,0.0122</t>
+  </si>
+  <si>
+    <t>0.7141,0.0364,0.2039,0.0653</t>
+  </si>
+  <si>
+    <t>0.9404,0.0580,0.0043,0.0054</t>
+  </si>
+  <si>
+    <t>0.9602,0.0461,0.0016,0.0037</t>
+  </si>
+  <si>
+    <t>0.9758,0.0264,0.0015,0.0030</t>
+  </si>
+  <si>
+    <t>0.9179,0.0892,0.0049,0.0057</t>
+  </si>
+  <si>
+    <t>0.9562,0.0438,0.0018,0.0053</t>
+  </si>
+  <si>
+    <t>0.9630,0.0351,0.0032,0.0044</t>
+  </si>
+  <si>
+    <t>0.9390,0.0744,0.0038,0.0051</t>
+  </si>
+  <si>
+    <t>0.9636,0.0335,0.0027,0.0056</t>
+  </si>
+  <si>
+    <t>0.0215,0.0291,0.9743,0.0031</t>
+  </si>
+  <si>
+    <t>0.0026,0.1286,0.9867,0.0010</t>
+  </si>
+  <si>
+    <t>0.0116,0.0282,0.9830,0.0020</t>
+  </si>
+  <si>
+    <t>0.1057,0.0106,0.9448,0.0029</t>
+  </si>
+  <si>
+    <t>0.0053,0.0205,0.9905,0.0023</t>
+  </si>
+  <si>
+    <t>0.1155,0.0070,0.9498,0.0058</t>
+  </si>
+  <si>
+    <t>0.1558,0.0166,0.9261,0.0032</t>
+  </si>
+  <si>
+    <t>0.0547,0.0062,0.9699,0.0040</t>
+  </si>
+  <si>
+    <t>0.7256,0.0089,0.0079,0.3608</t>
+  </si>
+  <si>
+    <t>0.1517,0.0878,0.0354,0.8743</t>
+  </si>
+  <si>
+    <t>0.0531,0.0139,0.0032,0.9778</t>
+  </si>
+  <si>
+    <t>0.0398,0.0098,0.0061,0.9799</t>
+  </si>
+  <si>
+    <t>0.0168,0.0127,0.0022,0.9910</t>
+  </si>
+  <si>
+    <t>0.7769,0.0386,0.0836,0.1077</t>
   </si>
 </sst>
 </file>
@@ -1967,7 +1967,7 @@
         <v>260</v>
       </c>
       <c r="C3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D3" t="s">
         <v>265</v>
@@ -2191,7 +2191,7 @@
         <v>262</v>
       </c>
       <c r="C19" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D19" t="s">
         <v>281</v>
@@ -2205,7 +2205,7 @@
         <v>262</v>
       </c>
       <c r="C20" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D20" t="s">
         <v>282</v>
@@ -2219,7 +2219,7 @@
         <v>262</v>
       </c>
       <c r="C21" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D21" t="s">
         <v>283</v>
@@ -2233,7 +2233,7 @@
         <v>262</v>
       </c>
       <c r="C22" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D22" t="s">
         <v>284</v>
@@ -2247,7 +2247,7 @@
         <v>262</v>
       </c>
       <c r="C23" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D23" t="s">
         <v>285</v>
@@ -2261,7 +2261,7 @@
         <v>259</v>
       </c>
       <c r="C24" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D24" t="s">
         <v>286</v>
@@ -2359,7 +2359,7 @@
         <v>259</v>
       </c>
       <c r="C31" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D31" t="s">
         <v>293</v>
@@ -2443,7 +2443,7 @@
         <v>259</v>
       </c>
       <c r="C37" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D37" t="s">
         <v>299</v>
@@ -2457,7 +2457,7 @@
         <v>262</v>
       </c>
       <c r="C38" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D38" t="s">
         <v>300</v>
@@ -2541,7 +2541,7 @@
         <v>262</v>
       </c>
       <c r="C44" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D44" t="s">
         <v>306</v>
@@ -2569,7 +2569,7 @@
         <v>259</v>
       </c>
       <c r="C46" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D46" t="s">
         <v>308</v>
@@ -2583,7 +2583,7 @@
         <v>262</v>
       </c>
       <c r="C47" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D47" t="s">
         <v>309</v>
@@ -2597,7 +2597,7 @@
         <v>262</v>
       </c>
       <c r="C48" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D48" t="s">
         <v>310</v>
@@ -2611,7 +2611,7 @@
         <v>262</v>
       </c>
       <c r="C49" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D49" t="s">
         <v>311</v>
@@ -2807,7 +2807,7 @@
         <v>262</v>
       </c>
       <c r="C63" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D63" t="s">
         <v>325</v>
@@ -2877,7 +2877,7 @@
         <v>262</v>
       </c>
       <c r="C68" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="D68" t="s">
         <v>330</v>
@@ -2947,7 +2947,7 @@
         <v>263</v>
       </c>
       <c r="C73" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D73" t="s">
         <v>335</v>
@@ -2961,7 +2961,7 @@
         <v>263</v>
       </c>
       <c r="C74" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D74" t="s">
         <v>336</v>
@@ -2975,7 +2975,7 @@
         <v>262</v>
       </c>
       <c r="C75" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D75" t="s">
         <v>337</v>
@@ -2989,7 +2989,7 @@
         <v>262</v>
       </c>
       <c r="C76" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D76" t="s">
         <v>338</v>
@@ -3003,7 +3003,7 @@
         <v>260</v>
       </c>
       <c r="C77" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D77" t="s">
         <v>339</v>
@@ -3017,7 +3017,7 @@
         <v>260</v>
       </c>
       <c r="C78" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D78" t="s">
         <v>340</v>
@@ -3031,7 +3031,7 @@
         <v>260</v>
       </c>
       <c r="C79" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D79" t="s">
         <v>341</v>
@@ -3045,7 +3045,7 @@
         <v>260</v>
       </c>
       <c r="C80" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D80" t="s">
         <v>342</v>
@@ -3059,7 +3059,7 @@
         <v>260</v>
       </c>
       <c r="C81" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D81" t="s">
         <v>343</v>
@@ -3073,7 +3073,7 @@
         <v>260</v>
       </c>
       <c r="C82" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D82" t="s">
         <v>344</v>
@@ -3087,7 +3087,7 @@
         <v>263</v>
       </c>
       <c r="C83" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D83" t="s">
         <v>345</v>
@@ -3115,7 +3115,7 @@
         <v>263</v>
       </c>
       <c r="C85" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D85" t="s">
         <v>347</v>
@@ -3143,7 +3143,7 @@
         <v>263</v>
       </c>
       <c r="C87" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D87" t="s">
         <v>349</v>
@@ -3157,7 +3157,7 @@
         <v>262</v>
       </c>
       <c r="C88" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D88" t="s">
         <v>350</v>
@@ -3423,7 +3423,7 @@
         <v>259</v>
       </c>
       <c r="C107" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D107" t="s">
         <v>369</v>
@@ -3451,7 +3451,7 @@
         <v>262</v>
       </c>
       <c r="C109" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D109" t="s">
         <v>371</v>
@@ -3465,7 +3465,7 @@
         <v>262</v>
       </c>
       <c r="C110" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D110" t="s">
         <v>372</v>
@@ -3479,7 +3479,7 @@
         <v>262</v>
       </c>
       <c r="C111" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D111" t="s">
         <v>373</v>
@@ -3493,7 +3493,7 @@
         <v>262</v>
       </c>
       <c r="C112" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D112" t="s">
         <v>374</v>
@@ -3507,7 +3507,7 @@
         <v>262</v>
       </c>
       <c r="C113" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D113" t="s">
         <v>375</v>
@@ -3521,7 +3521,7 @@
         <v>262</v>
       </c>
       <c r="C114" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D114" t="s">
         <v>376</v>
@@ -3535,7 +3535,7 @@
         <v>262</v>
       </c>
       <c r="C115" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D115" t="s">
         <v>377</v>
@@ -3577,7 +3577,7 @@
         <v>259</v>
       </c>
       <c r="C118" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D118" t="s">
         <v>380</v>
@@ -3605,7 +3605,7 @@
         <v>262</v>
       </c>
       <c r="C120" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D120" t="s">
         <v>382</v>
@@ -3619,7 +3619,7 @@
         <v>262</v>
       </c>
       <c r="C121" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D121" t="s">
         <v>383</v>
@@ -3633,7 +3633,7 @@
         <v>262</v>
       </c>
       <c r="C122" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D122" t="s">
         <v>384</v>
@@ -3647,7 +3647,7 @@
         <v>262</v>
       </c>
       <c r="C123" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D123" t="s">
         <v>385</v>
@@ -3661,7 +3661,7 @@
         <v>263</v>
       </c>
       <c r="C124" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D124" t="s">
         <v>386</v>
@@ -3675,7 +3675,7 @@
         <v>262</v>
       </c>
       <c r="C125" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D125" t="s">
         <v>387</v>
@@ -3703,7 +3703,7 @@
         <v>259</v>
       </c>
       <c r="C127" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D127" t="s">
         <v>389</v>
@@ -3885,7 +3885,7 @@
         <v>259</v>
       </c>
       <c r="C140" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D140" t="s">
         <v>402</v>
@@ -3899,7 +3899,7 @@
         <v>259</v>
       </c>
       <c r="C141" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D141" t="s">
         <v>403</v>
@@ -3927,7 +3927,7 @@
         <v>259</v>
       </c>
       <c r="C143" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D143" t="s">
         <v>405</v>
@@ -3941,7 +3941,7 @@
         <v>260</v>
       </c>
       <c r="C144" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D144" t="s">
         <v>406</v>
@@ -3955,7 +3955,7 @@
         <v>260</v>
       </c>
       <c r="C145" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D145" t="s">
         <v>407</v>
@@ -3969,7 +3969,7 @@
         <v>260</v>
       </c>
       <c r="C146" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D146" t="s">
         <v>408</v>
@@ -3983,7 +3983,7 @@
         <v>260</v>
       </c>
       <c r="C147" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D147" t="s">
         <v>409</v>
@@ -4025,7 +4025,7 @@
         <v>262</v>
       </c>
       <c r="C150" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D150" t="s">
         <v>412</v>
@@ -4347,7 +4347,7 @@
         <v>259</v>
       </c>
       <c r="C173" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D173" t="s">
         <v>435</v>
@@ -4361,7 +4361,7 @@
         <v>259</v>
       </c>
       <c r="C174" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D174" t="s">
         <v>436</v>
@@ -4375,7 +4375,7 @@
         <v>262</v>
       </c>
       <c r="C175" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D175" t="s">
         <v>437</v>
@@ -4669,7 +4669,7 @@
         <v>259</v>
       </c>
       <c r="C196" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D196" t="s">
         <v>458</v>
@@ -4683,7 +4683,7 @@
         <v>259</v>
       </c>
       <c r="C197" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D197" t="s">
         <v>459</v>
@@ -4697,7 +4697,7 @@
         <v>259</v>
       </c>
       <c r="C198" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D198" t="s">
         <v>460</v>
@@ -4711,7 +4711,7 @@
         <v>262</v>
       </c>
       <c r="C199" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D199" t="s">
         <v>461</v>
@@ -4725,7 +4725,7 @@
         <v>262</v>
       </c>
       <c r="C200" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D200" t="s">
         <v>462</v>
@@ -4753,7 +4753,7 @@
         <v>259</v>
       </c>
       <c r="C202" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D202" t="s">
         <v>464</v>
@@ -4795,7 +4795,7 @@
         <v>259</v>
       </c>
       <c r="C205" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D205" t="s">
         <v>467</v>
@@ -5033,7 +5033,7 @@
         <v>259</v>
       </c>
       <c r="C222" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D222" t="s">
         <v>484</v>
@@ -5411,7 +5411,7 @@
         <v>261</v>
       </c>
       <c r="C249" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D249" t="s">
         <v>511</v>
@@ -5453,7 +5453,7 @@
         <v>260</v>
       </c>
       <c r="C252" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D252" t="s">
         <v>514</v>
@@ -5467,7 +5467,7 @@
         <v>260</v>
       </c>
       <c r="C253" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D253" t="s">
         <v>515</v>
@@ -5481,7 +5481,7 @@
         <v>260</v>
       </c>
       <c r="C254" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D254" t="s">
         <v>516</v>
@@ -5495,7 +5495,7 @@
         <v>260</v>
       </c>
       <c r="C255" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D255" t="s">
         <v>517</v>

</xml_diff>